<commit_message>
save 03 06 2026
</commit_message>
<xml_diff>
--- a/4 четверть_10_JavaScript_MoleculerJS.xlsx
+++ b/4 четверть_10_JavaScript_MoleculerJS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C7D1060-B713-4880-B659-DFE72A54060F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3835F27E-9E95-479A-94BF-2A1D3CD88AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7515" yWindow="-18705" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Basics" sheetId="12" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1835" uniqueCount="1532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1846" uniqueCount="1541">
   <si>
     <t>Документация https://moleculer.services/docs/0.14/broker</t>
   </si>
@@ -18089,17 +18089,228 @@
       <t>broadcast</t>
     </r>
   </si>
+  <si>
+    <t>Environment variables
+My experience</t>
+  </si>
+  <si>
+    <t>package.json</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">{
+  "name": "lk2-prod-back",
+  "version": "1.0.0",
+  "main": "index.js",
+  "license": "MIT",
+  "scripts": {
+    "prod": "set PROD=true &amp;&amp; nodemon index.js",
+    "start": "set PROD=true &amp;&amp; node --max_old_space_size=8000 index.js",
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"dev": "set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NODE_ENV=development&amp;&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> node --inspect=localhost:9230 --max_old_space_size=8000 index.js",
+    "auth": "set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NODE_ENV=auth&amp;&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> node --inspect=localhost:9230 --max_old_space_size=8000 index.js"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  },
+  "dependencies": {
+    "apicache": "1.5.2",
+    "app-root-path": "^2.2.1",
+    "axios": "^1.13.5",
+    "basic-ftp": "^5.1.0",
+    "clickhouse": "^2.6.0",
+    "colors": "^1.4.0",
+    "connect-timeout": "^1.9.1",
+    "cookie-parser": "^1.4.7",
+    "crypto-js": "^3.3.0",
+    "cyrillic-to-translit-js": "^3.2.1",
+    "dotenv": "^16.6.1",</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Объявить в скрипте:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+set NODE_ENV=development&amp;&amp;</t>
+    </r>
+  </si>
+  <si>
+    <t>Файлы .env</t>
+  </si>
+  <si>
+    <t>env.development</t>
+  </si>
+  <si>
+    <t>AUTH_PORT=4040
+FOLDER_EXCEL_EXE=2
+AUTH=0
+LOCAL_AUTH_BYPASS_TOKEN=eyJhbGciOiJSUzI1NiIsInR5cCI6IkpXVCJ9.eyJpcCI6IjEyNy4wLjAuMSIsIklkVXNlciI6NjQwNTgsInVzZXJJZCI6IlN1cGVyVXNlckBzdWRvLnJ1IiwiSWRVc2VyVHlwZSI6MSwidXNlckRpcmVjdG9yeSI6IlN1cGVyVXNlckNvbXBhbnkiLCJMaWNlbnNlQ29uZmlybSI6IjIwMjYtMDUtMjdUMTI6Mzc6MTIuODEwIiwiUGVyc29uYWxEYXRhQ29uZmlybSI6IjIwMjYtMDUtMjdUMTQ6MDA6NTYuMzUwIiwiVGVsZWdyYW1DaGF0IjpudWxsLCJVc2VySGFzVG90cCI6ZmFsc2UsIlVzZXJNYWlsUmVzZXJ2ZUZvclRmYSI6bnVsbCwiVGZhQWN0aXZlIjpmYWxzZSwiVXNlckNvbXBhbnkiOnsiQ29tcGFueU5hbWUiOiJTdXBlclVzZXJDb21wYW55IiwiSWRDb21wYW55TWFuYWdlciI6NjI4NzcsIk1lc3NhZ2Vyc09mZkJ5QWRtIjpmYWxzZX0sIk1heENoYXRJZCI6bnVsbCwibW9kZSI6InVzZXIiLCJVSUQiOiJ0cjk2MTBnc2hjOHR3Zm9oMW1za2ciLCJJZE1hbmFnZXIiOm51bGwsImJpSWQiOjAsImJpRW1haWwiOiJTdXBlclVzZXJAc3Vkby5ydSIsImJpVHlwZSI6Imd1ZXN0IiwiaWF0IjoxNzc5ODg2MDE1fQ.WAsHJINIKgkHtWKBlL-psoTB4q8E2y4Cwf8NpsSV03Cq6c6NpeC-BQe9a4Pf53ZxFeT49SJQhIE3S2eVFIBU01cqbfutqqc2gU8C2WvQz2xjkXDCw_jTqVw8qyJ04ycW9ENqnOeaS7r-6FuOGuC3MOkButRCifgMba7EMUTVSygyDgxeJFV6g0cMtKNPD5QfxskE2AUFEXM6retypuMKw7nM3WxkzAaBI_Pom2Mb9UUr5ogDdF9i1MDhYzx5ZLFAkx-WFC1LeS9rclp4Ja9JmdldDFW__OdwSd3m-CSzG9JSPfoThHXB7WRmaFe78HBEdBafwU553QDpgUuSGOtxX048N0PIo3chPixkzdg7l4A2134XzsGb4a4u8UhuvFXuk_srfh1RpwLxmLsxlASgj0PS8ikOaN6W8eQHgFQK2jRB3yAUoQYnzwZgQvloontnRQdXdeOjkIIdPswhrsl7xnj2EGEmJIZxjIkGoUPx1IMxf-itycFvqUO5NYVAH7rygIldCHdjXb99r5uwyfrYSkMHqATfe4mjguhay9sIUPB2iMnzSWp8mgjjy8yAJqed676a9gmDC7hq5kzHVSWhuTRdD8D5qauY57yHtxDV005qvV9DPCMjGw9sqEra1urKVCMcyeCzrBVJOwewvrwgBAGHWj9Myy6QHi9fZtmSDNE
+ALLOW_LOCAL_AUTH_BYPASS=true</t>
+  </si>
+  <si>
+    <t>Вызов переменных окружения</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">const tokens = require('./tokens');
+module.exports = {
+  baseURL: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>+process.env.AUTH</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ? `http://127.0.0.1:${</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>process.env.AUTH_PORT.trim()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>}/api` : `http://10.233.233.110:${process.env.AUTH_PORT.trim()}/api`,
+  timeout: 10000,
+  headers: {'innerauth': 'Server ' + tokens.lk},
+};</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="45">
+  <fonts count="46">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -18767,7 +18978,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -18778,23 +18989,23 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -18812,7 +19023,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -18830,7 +19041,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -18851,7 +19062,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -18872,7 +19083,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -18890,10 +19101,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -18902,28 +19113,28 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -18932,49 +19143,49 @@
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -18983,7 +19194,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -18992,7 +19203,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19004,7 +19215,7 @@
     <xf numFmtId="49" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19013,22 +19224,22 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19040,89 +19251,92 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -19130,28 +19344,28 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -19233,7 +19447,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>324715</xdr:rowOff>
+      <xdr:rowOff>320905</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -19317,14 +19531,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>132310</xdr:rowOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>136120</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -19365,14 +19579,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>144779</xdr:colOff>
-      <xdr:row>69</xdr:row>
+      <xdr:row>76</xdr:row>
       <xdr:rowOff>163157</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>3350893</xdr:colOff>
-      <xdr:row>69</xdr:row>
-      <xdr:rowOff>1617345</xdr:rowOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>1621155</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -20624,7 +20838,7 @@
       <c r="D27" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -25905,7 +26119,7 @@
       <c r="V87" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -27789,7 +28003,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V70"/>
+  <dimension ref="A2:V77"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -28170,224 +28384,279 @@
         <v>563</v>
       </c>
     </row>
+    <row r="38" spans="1:4" ht="28.8">
+      <c r="A38" s="63" t="s">
+        <v>1532</v>
+      </c>
+      <c r="B38" s="52"/>
+      <c r="C38" s="52"/>
+    </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="3"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="3"/>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="C40" s="69" t="s">
+      <c r="A39" s="47" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B39" s="130" t="s">
+        <v>580</v>
+      </c>
+      <c r="C39" s="52"/>
+    </row>
+    <row r="40" spans="1:4" ht="360">
+      <c r="B40" s="130" t="s">
+        <v>1535</v>
+      </c>
+      <c r="C40" s="130" t="s">
+        <v>1534</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="47" t="s">
+        <v>1536</v>
+      </c>
+      <c r="B41" s="130" t="s">
+        <v>581</v>
+      </c>
+      <c r="C41" s="52"/>
+    </row>
+    <row r="42" spans="1:4" ht="403.2">
+      <c r="A42" s="1" t="s">
+        <v>1537</v>
+      </c>
+      <c r="B42" s="52"/>
+      <c r="C42" s="130" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="47" t="s">
+        <v>1539</v>
+      </c>
+      <c r="B43" s="52"/>
+      <c r="C43" s="52"/>
+    </row>
+    <row r="44" spans="1:4" ht="129.6">
+      <c r="B44" s="52"/>
+      <c r="C44" s="130" t="s">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="3"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="3"/>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="C47" s="69" t="s">
         <v>793</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="12" t="s">
+    <row r="48" spans="1:4">
+      <c r="A48" s="12" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="28.8">
-      <c r="C42" s="68" t="s">
+    <row r="49" spans="1:4" ht="28.8">
+      <c r="C49" s="68" t="s">
         <v>794</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="28.8">
-      <c r="C43" s="68" t="s">
+    <row r="50" spans="1:4" ht="28.8">
+      <c r="C50" s="68" t="s">
         <v>795</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="13" t="s">
+    <row r="51" spans="1:4">
+      <c r="A51" s="13" t="s">
         <v>819</v>
-      </c>
-      <c r="B44" s="55" t="s">
-        <v>796</v>
-      </c>
-      <c r="C44" s="68"/>
-      <c r="D44" s="1" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="403.2">
-      <c r="B45" s="2" t="s">
-        <v>821</v>
-      </c>
-      <c r="C45" s="68" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4">
-      <c r="A46" s="13" t="s">
-        <v>823</v>
-      </c>
-      <c r="B46" s="55" t="s">
-        <v>796</v>
-      </c>
-      <c r="C46" s="68"/>
-      <c r="D46" s="1" t="s">
-        <v>829</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="409.6">
-      <c r="C47" s="68" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4">
-      <c r="A48" s="13" t="s">
-        <v>824</v>
-      </c>
-      <c r="B48" s="55" t="s">
-        <v>796</v>
-      </c>
-      <c r="C48" s="68"/>
-      <c r="D48" s="1" t="s">
-        <v>828</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="316.8">
-      <c r="B49" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="C49" s="68" t="s">
-        <v>827</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4">
-      <c r="A50" s="13" t="s">
-        <v>803</v>
-      </c>
-      <c r="C50" s="68"/>
-      <c r="D50" s="1" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4">
-      <c r="A51" s="85" t="s">
-        <v>799</v>
       </c>
       <c r="B51" s="55" t="s">
         <v>796</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" ht="331.2">
+      <c r="C51" s="68"/>
+      <c r="D51" s="1" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="403.2">
+      <c r="B52" s="2" t="s">
+        <v>821</v>
+      </c>
       <c r="C52" s="68" t="s">
-        <v>801</v>
+        <v>822</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="13" t="s">
+        <v>823</v>
+      </c>
+      <c r="B53" s="55" t="s">
+        <v>796</v>
+      </c>
+      <c r="C53" s="68"/>
+      <c r="D53" s="1" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="409.6">
+      <c r="C54" s="68" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="13" t="s">
+        <v>824</v>
+      </c>
+      <c r="B55" s="55" t="s">
+        <v>796</v>
+      </c>
+      <c r="C55" s="68"/>
+      <c r="D55" s="1" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="316.8">
+      <c r="B56" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="C56" s="68" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="13" t="s">
+        <v>803</v>
+      </c>
+      <c r="C57" s="68"/>
+      <c r="D57" s="1" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="85" t="s">
+        <v>799</v>
+      </c>
+      <c r="B58" s="55" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="331.2">
+      <c r="C59" s="68" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="13" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="28.8">
-      <c r="B54" s="55" t="s">
+    <row r="61" spans="1:4" ht="28.8">
+      <c r="B61" s="55" t="s">
         <v>796</v>
       </c>
-      <c r="C54" s="68" t="s">
+      <c r="C61" s="68" t="s">
         <v>805</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="28.8">
-      <c r="A55" s="85" t="s">
+    <row r="62" spans="1:4" ht="28.8">
+      <c r="A62" s="85" t="s">
         <v>800</v>
       </c>
-      <c r="B55" s="1"/>
-      <c r="C55" s="68"/>
-    </row>
-    <row r="56" spans="1:4" ht="43.2">
-      <c r="B56" s="2" t="s">
+      <c r="B62" s="1"/>
+      <c r="C62" s="68"/>
+    </row>
+    <row r="63" spans="1:4" ht="43.2">
+      <c r="B63" s="2" t="s">
         <v>806</v>
       </c>
-      <c r="C56" s="68" t="s">
+      <c r="C63" s="68" t="s">
         <v>811</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
-      <c r="A57" s="85" t="s">
+    <row r="64" spans="1:4">
+      <c r="A64" s="85" t="s">
         <v>799</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="316.8">
-      <c r="C58" s="68" t="s">
+    <row r="65" spans="1:4" ht="316.8">
+      <c r="C65" s="68" t="s">
         <v>810</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
-      <c r="A59" s="13" t="s">
+    <row r="66" spans="1:4">
+      <c r="A66" s="13" t="s">
         <v>808</v>
       </c>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1" t="s">
+      <c r="B66" s="1"/>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1" t="s">
         <v>807</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="28.8">
-      <c r="B60" s="55" t="s">
+    <row r="67" spans="1:4" ht="28.8">
+      <c r="B67" s="55" t="s">
         <v>796</v>
       </c>
-      <c r="C60" s="68" t="s">
+      <c r="C67" s="68" t="s">
         <v>813</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="28.8">
-      <c r="A61" s="85" t="s">
+    <row r="68" spans="1:4" ht="28.8">
+      <c r="A68" s="85" t="s">
         <v>800</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="43.2">
-      <c r="C62" s="68" t="s">
+    <row r="69" spans="1:4" ht="43.2">
+      <c r="C69" s="68" t="s">
         <v>809</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
-      <c r="A63" s="85" t="s">
+    <row r="70" spans="1:4">
+      <c r="A70" s="85" t="s">
         <v>799</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="273.60000000000002">
-      <c r="C64" s="68" t="s">
+    <row r="71" spans="1:4" ht="273.60000000000002">
+      <c r="C71" s="68" t="s">
         <v>812</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
-      <c r="A65" s="13" t="s">
+    <row r="72" spans="1:4">
+      <c r="A72" s="13" t="s">
         <v>814</v>
       </c>
-      <c r="D65" s="1" t="s">
+      <c r="D72" s="1" t="s">
         <v>815</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="43.2">
-      <c r="B66" s="55" t="s">
+    <row r="73" spans="1:4" ht="43.2">
+      <c r="B73" s="55" t="s">
         <v>796</v>
       </c>
-      <c r="C66" s="68" t="s">
+      <c r="C73" s="68" t="s">
         <v>816</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="28.8">
-      <c r="A67" s="85" t="s">
+    <row r="74" spans="1:4" ht="28.8">
+      <c r="A74" s="85" t="s">
         <v>800</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="43.2">
-      <c r="C68" s="68" t="s">
+    <row r="75" spans="1:4" ht="43.2">
+      <c r="C75" s="68" t="s">
         <v>817</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
-      <c r="A69" s="85" t="s">
+    <row r="76" spans="1:4">
+      <c r="A76" s="85" t="s">
         <v>799</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="345.6">
-      <c r="B70"/>
-      <c r="C70" s="68" t="s">
+    <row r="77" spans="1:4" ht="345.6">
+      <c r="B77"/>
+      <c r="C77" s="68" t="s">
         <v>818</v>
       </c>
     </row>

</xml_diff>

<commit_message>
save 05 06 2026
</commit_message>
<xml_diff>
--- a/4 четверть_10_JavaScript_MoleculerJS.xlsx
+++ b/4 четверть_10_JavaScript_MoleculerJS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3835F27E-9E95-479A-94BF-2A1D3CD88AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794015C9-93E3-4C31-A3FE-1853ADAAA99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7515" yWindow="-18705" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="15" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Basics" sheetId="12" r:id="rId1"/>
@@ -29,10 +29,10 @@
     <sheet name="ctx" sheetId="22" r:id="rId14"/>
     <sheet name="Service (ES6)" sheetId="20" r:id="rId15"/>
     <sheet name="API Gateway" sheetId="18" r:id="rId16"/>
-    <sheet name="File up(down)load aliases" sheetId="35" r:id="rId17"/>
-    <sheet name="Response type" sheetId="36" r:id="rId18"/>
-    <sheet name="Authorization &amp; Authent" sheetId="37" r:id="rId19"/>
-    <sheet name="Extras" sheetId="38" r:id="rId20"/>
+    <sheet name="Hooks" sheetId="38" r:id="rId17"/>
+    <sheet name="File up(down)load aliases" sheetId="35" r:id="rId18"/>
+    <sheet name="Response type" sheetId="36" r:id="rId19"/>
+    <sheet name="Authorization &amp; Authent" sheetId="37" r:id="rId20"/>
     <sheet name="Transporter" sheetId="31" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1846" uniqueCount="1541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="1542">
   <si>
     <t>Документация https://moleculer.services/docs/0.14/broker</t>
   </si>
@@ -18292,17 +18292,50 @@
 };</t>
     </r>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Важно! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>В Moleculer API Gateway есть строгий контракт для кастомного хранилища - методы должны называться именно inc() и reset() (или clear()).</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="46">
+  <fonts count="47">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -18978,7 +19011,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -18989,23 +19022,23 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -19023,7 +19056,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19041,7 +19074,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19062,7 +19095,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19083,7 +19116,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19101,10 +19134,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19113,28 +19146,28 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19143,49 +19176,49 @@
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19194,7 +19227,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19203,7 +19236,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19215,7 +19248,7 @@
     <xf numFmtId="49" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19224,22 +19257,22 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19251,89 +19284,92 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -19341,28 +19377,28 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -20838,7 +20874,7 @@
       <c r="D27" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="20" type="noConversion"/>
+  <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -26119,13 +26155,319 @@
       <c r="V87" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="20" type="noConversion"/>
+  <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{215A08A6-8FA5-47FE-AD3E-099EDF44B417}">
+  <sheetPr>
+    <tabColor theme="4" tint="-0.249977111117893"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V40"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="41.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3" s="116" t="s">
+        <v>1468</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22">
+      <c r="C4" s="115" t="s">
+        <v>1469</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22">
+      <c r="C5" s="115" t="s">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22">
+      <c r="C6" s="115" t="s">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22">
+      <c r="C7" s="115" t="s">
+        <v>1303</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22">
+      <c r="C8" s="115" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22">
+      <c r="C9" s="115" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>1497</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22">
+      <c r="C10" s="115" t="s">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22">
+      <c r="C11" s="115" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
+      <c r="A13" s="118" t="s">
+        <v>1469</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="28.8">
+      <c r="C14" s="115" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="302.39999999999998">
+      <c r="C15" s="115" t="s">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22">
+      <c r="A16" s="12" t="s">
+        <v>1470</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>1477</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="C17" s="115" t="s">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="331.2">
+      <c r="B18" s="2" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C18" s="115" t="s">
+        <v>1481</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="12" t="s">
+        <v>1302</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>1478</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="28.8">
+      <c r="C20" s="115" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="302.39999999999998">
+      <c r="C21" s="115" t="s">
+        <v>1485</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="172.8">
+      <c r="C22" s="115" t="s">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="12" t="s">
+        <v>1303</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="409.6">
+      <c r="A24" s="131" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>1488</v>
+      </c>
+      <c r="C24" s="131" t="s">
+        <v>1487</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="129.6">
+      <c r="B26" s="2" t="s">
+        <v>1494</v>
+      </c>
+      <c r="C26" s="115" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="230.4">
+      <c r="B27" s="2" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C27" s="115" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>1493</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="12" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>1497</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="28.8">
+      <c r="C29" s="115" t="s">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="244.8">
+      <c r="C30" s="115" t="s">
+        <v>1495</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="12" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C31" s="1"/>
+    </row>
+    <row r="32" spans="1:4" ht="43.2">
+      <c r="A32" s="2"/>
+      <c r="C32" s="115" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="86.4">
+      <c r="A33" s="2" t="s">
+        <v>1506</v>
+      </c>
+      <c r="C33" s="115" t="s">
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="2"/>
+      <c r="C34" s="115"/>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="119" t="s">
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="C36" s="115" t="s">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="13" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="129.6">
+      <c r="C38" s="115" t="s">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="244.8">
+      <c r="A39" s="1" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C39" s="115" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="288">
+      <c r="A40" s="1" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C40" s="115" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E63D7CF-A8C1-4EE2-B24F-BB6423312324}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -26267,7 +26609,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0E1A7F4-4156-43BA-A471-45FED5CB2B12}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -26407,140 +26749,6 @@
       </c>
       <c r="C13" s="120" t="s">
         <v>1455</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC0D01A-891F-4564-985B-BABA4F41741B}">
-  <sheetPr>
-    <tabColor theme="4" tint="-0.249977111117893"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A2:V12"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="41.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" style="8"/>
-    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.77734375" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:22">
-      <c r="A2" s="3"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="U2" s="5"/>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="C3" s="116" t="s">
-        <v>1463</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>1461</v>
-      </c>
-      <c r="P3" s="1"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:22">
-      <c r="A4" s="12" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22">
-      <c r="C5" s="115" t="s">
-        <v>1456</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22" ht="43.2">
-      <c r="B6" s="121" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C6" s="121" t="s">
-        <v>1457</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22" ht="172.8">
-      <c r="C7" s="121" t="s">
-        <v>1458</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22" ht="403.2">
-      <c r="B8" s="2" t="s">
-        <v>1460</v>
-      </c>
-      <c r="C8" s="115" t="s">
-        <v>1459</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22">
-      <c r="A9" s="12" t="s">
-        <v>1462</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>1464</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" ht="28.8">
-      <c r="C10" s="115" t="s">
-        <v>1465</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22" ht="43.2">
-      <c r="B11" s="121" t="s">
-        <v>1512</v>
-      </c>
-      <c r="C11" s="121" t="s">
-        <v>1466</v>
-      </c>
-    </row>
-    <row r="12" spans="1:22" ht="409.6">
-      <c r="C12" s="115" t="s">
-        <v>1467</v>
       </c>
     </row>
   </sheetData>
@@ -26665,12 +26873,12 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{215A08A6-8FA5-47FE-AD3E-099EDF44B417}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC0D01A-891F-4564-985B-BABA4F41741B}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V40"/>
+  <dimension ref="A2:V12"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="41.33203125" style="1" customWidth="1"/>
@@ -26726,239 +26934,70 @@
         <v>300</v>
       </c>
       <c r="C3" s="116" t="s">
-        <v>1468</v>
+        <v>1463</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>1461</v>
       </c>
       <c r="P3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="2"/>
     </row>
     <row r="4" spans="1:22">
-      <c r="C4" s="115" t="s">
-        <v>1469</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>1476</v>
+      <c r="A4" s="12" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="5" spans="1:22">
       <c r="C5" s="115" t="s">
-        <v>1470</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22">
-      <c r="C6" s="115" t="s">
-        <v>1302</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22">
-      <c r="C7" s="115" t="s">
-        <v>1303</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22">
+        <v>1456</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="43.2">
+      <c r="B6" s="121" t="s">
+        <v>1511</v>
+      </c>
+      <c r="C6" s="121" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="172.8">
+      <c r="C7" s="121" t="s">
+        <v>1458</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="403.2">
+      <c r="B8" s="2" t="s">
+        <v>1460</v>
+      </c>
       <c r="C8" s="115" t="s">
-        <v>1471</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="9" spans="1:22">
-      <c r="C9" s="115" t="s">
-        <v>1472</v>
+      <c r="A9" s="12" t="s">
+        <v>1462</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>1497</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="28.8">
       <c r="C10" s="115" t="s">
-        <v>1473</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22">
-      <c r="C11" s="115" t="s">
-        <v>1474</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>1475</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22">
-      <c r="A13" s="118" t="s">
-        <v>1469</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>1476</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22" ht="28.8">
-      <c r="C14" s="115" t="s">
-        <v>1479</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" ht="302.39999999999998">
-      <c r="C15" s="115" t="s">
-        <v>1482</v>
-      </c>
-    </row>
-    <row r="16" spans="1:22">
-      <c r="A16" s="12" t="s">
-        <v>1470</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>1477</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="C17" s="115" t="s">
-        <v>1480</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="331.2">
-      <c r="B18" s="2" t="s">
-        <v>1483</v>
-      </c>
-      <c r="C18" s="115" t="s">
-        <v>1481</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="12" t="s">
-        <v>1302</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>1478</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="28.8">
-      <c r="C20" s="115" t="s">
-        <v>1484</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="302.39999999999998">
-      <c r="C21" s="115" t="s">
-        <v>1485</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="172.8">
-      <c r="C22" s="115" t="s">
-        <v>1486</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="12" t="s">
-        <v>1303</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="409.6">
-      <c r="B24" s="2" t="s">
-        <v>1488</v>
-      </c>
-      <c r="C24" s="115" t="s">
-        <v>1487</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="12" t="s">
-        <v>1471</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>1491</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="129.6">
-      <c r="B26" s="2" t="s">
-        <v>1494</v>
-      </c>
-      <c r="C26" s="115" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="230.4">
-      <c r="B27" s="2" t="s">
-        <v>1492</v>
-      </c>
-      <c r="C27" s="115" t="s">
-        <v>1490</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>1493</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="12" t="s">
-        <v>1472</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>1497</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="28.8">
-      <c r="C29" s="115" t="s">
-        <v>1496</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="244.8">
-      <c r="C30" s="115" t="s">
-        <v>1495</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="12" t="s">
-        <v>1498</v>
-      </c>
-      <c r="C31" s="1"/>
-    </row>
-    <row r="32" spans="1:4" ht="43.2">
-      <c r="A32" s="2"/>
-      <c r="C32" s="115" t="s">
-        <v>1505</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="86.4">
-      <c r="A33" s="2" t="s">
-        <v>1506</v>
-      </c>
-      <c r="C33" s="115" t="s">
-        <v>1507</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="2"/>
-      <c r="C34" s="115"/>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" s="119" t="s">
-        <v>1316</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="C36" s="115" t="s">
-        <v>1499</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" s="13" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="129.6">
-      <c r="C38" s="115" t="s">
-        <v>1501</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="244.8">
-      <c r="A39" s="1" t="s">
-        <v>1502</v>
-      </c>
-      <c r="C39" s="115" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="288">
-      <c r="A40" s="1" t="s">
-        <v>1504</v>
-      </c>
-      <c r="C40" s="115" t="s">
-        <v>1500</v>
+        <v>1465</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="43.2">
+      <c r="B11" s="121" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C11" s="121" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" ht="409.6">
+      <c r="C12" s="115" t="s">
+        <v>1467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
save 08 07 2026
</commit_message>
<xml_diff>
--- a/4 четверть_10_JavaScript_MoleculerJS.xlsx
+++ b/4 четверть_10_JavaScript_MoleculerJS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794015C9-93E3-4C31-A3FE-1853ADAAA99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48406B57-E8AC-42A3-B3DD-AD9399AE7576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="15" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Basics" sheetId="12" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="1542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1849" uniqueCount="1543">
   <si>
     <t>Документация https://moleculer.services/docs/0.14/broker</t>
   </si>
@@ -18238,7 +18238,53 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">const tokens = require('./tokens');
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Важно! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>В Moleculer API Gateway есть строгий контракт для кастомного хранилища - методы должны называться именно inc() и reset() (или clear()).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>require('dotenv').config({ path: `.env.${process.env.NODE_ENV}`});</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+const tokens = require('./tokens');
 module.exports = {
   baseURL: </t>
     </r>
@@ -18293,41 +18339,27 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Важно! </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>В Moleculer API Gateway есть строгий контракт для кастомного хранилища - методы должны называться именно inc() и reset() (или clear()).</t>
-    </r>
+    <t>dotenv - https://www.npmjs.com/package/dotenv</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="47">
+  <fonts count="48">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -19011,7 +19043,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -19022,23 +19054,23 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -19056,7 +19088,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19074,7 +19106,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19095,7 +19127,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19116,7 +19148,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19134,10 +19166,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19146,28 +19178,28 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19176,49 +19208,49 @@
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="31" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="30" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="31" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19227,7 +19259,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19236,7 +19268,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19248,7 +19280,7 @@
     <xf numFmtId="49" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19257,22 +19289,22 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19284,89 +19316,92 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="31" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -19374,28 +19409,28 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -19574,7 +19609,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>48</xdr:row>
-      <xdr:rowOff>136120</xdr:rowOff>
+      <xdr:rowOff>136121</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -20874,7 +20909,7 @@
       <c r="D27" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -26155,7 +26190,7 @@
       <c r="V87" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -26347,7 +26382,7 @@
     </row>
     <row r="24" spans="1:4" ht="409.6">
       <c r="A24" s="131" t="s">
-        <v>1541</v>
+        <v>1540</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>1488</v>
@@ -28437,7 +28472,9 @@
       <c r="B39" s="130" t="s">
         <v>580</v>
       </c>
-      <c r="C39" s="52"/>
+      <c r="C39" s="132" t="s">
+        <v>1542</v>
+      </c>
     </row>
     <row r="40" spans="1:4" ht="360">
       <c r="B40" s="130" t="s">
@@ -28457,7 +28494,7 @@
       <c r="C41" s="52"/>
     </row>
     <row r="42" spans="1:4" ht="403.2">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="67" t="s">
         <v>1537</v>
       </c>
       <c r="B42" s="52"/>
@@ -28469,13 +28506,15 @@
       <c r="A43" s="47" t="s">
         <v>1539</v>
       </c>
-      <c r="B43" s="52"/>
+      <c r="B43" s="132" t="s">
+        <v>582</v>
+      </c>
       <c r="C43" s="52"/>
     </row>
-    <row r="44" spans="1:4" ht="129.6">
+    <row r="44" spans="1:4" ht="144">
       <c r="B44" s="52"/>
-      <c r="C44" s="130" t="s">
-        <v>1540</v>
+      <c r="C44" s="132" t="s">
+        <v>1541</v>
       </c>
     </row>
     <row r="46" spans="1:4">

</xml_diff>

<commit_message>
save 13 07 2026
</commit_message>
<xml_diff>
--- a/4 четверть_10_JavaScript_MoleculerJS.xlsx
+++ b/4 четверть_10_JavaScript_MoleculerJS.xlsx
@@ -8,32 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48406B57-E8AC-42A3-B3DD-AD9399AE7576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC03B171-CC95-46F3-9DA5-2C45E5DAA4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4470" yWindow="-18225" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Basics" sheetId="12" r:id="rId1"/>
-    <sheet name="init new proj" sheetId="15" r:id="rId2"/>
-    <sheet name="MoleculerError (Controller)" sheetId="33" r:id="rId3"/>
-    <sheet name="SB, config.js, env, Logging" sheetId="19" r:id="rId4"/>
-    <sheet name="ServiceBroker" sheetId="13" r:id="rId5"/>
-    <sheet name="Service" sheetId="17" r:id="rId6"/>
-    <sheet name="mixins{}" sheetId="30" r:id="rId7"/>
-    <sheet name="events{}" sheetId="27" r:id="rId8"/>
-    <sheet name="LCevents" sheetId="28" r:id="rId9"/>
-    <sheet name="act hooks{}" sheetId="26" r:id="rId10"/>
-    <sheet name="Middleware" sheetId="24" r:id="rId11"/>
-    <sheet name="act caching" sheetId="32" r:id="rId12"/>
-    <sheet name="settings{}depend()" sheetId="29" r:id="rId13"/>
-    <sheet name="ctx" sheetId="22" r:id="rId14"/>
-    <sheet name="Service (ES6)" sheetId="20" r:id="rId15"/>
-    <sheet name="API Gateway" sheetId="18" r:id="rId16"/>
-    <sheet name="Hooks" sheetId="38" r:id="rId17"/>
-    <sheet name="File up(down)load aliases" sheetId="35" r:id="rId18"/>
-    <sheet name="Response type" sheetId="36" r:id="rId19"/>
-    <sheet name="Authorization &amp; Authent" sheetId="37" r:id="rId20"/>
-    <sheet name="Transporter" sheetId="31" r:id="rId21"/>
+    <sheet name="Для изучения" sheetId="40" r:id="rId1"/>
+    <sheet name="Basics" sheetId="12" r:id="rId2"/>
+    <sheet name="init new proj" sheetId="15" r:id="rId3"/>
+    <sheet name="Proj architecture" sheetId="39" r:id="rId4"/>
+    <sheet name="MoleculerError (Controller)" sheetId="33" r:id="rId5"/>
+    <sheet name="SB, config.js, env, Logging" sheetId="19" r:id="rId6"/>
+    <sheet name="ServiceBroker" sheetId="13" r:id="rId7"/>
+    <sheet name="Service" sheetId="17" r:id="rId8"/>
+    <sheet name="mixins{}" sheetId="30" r:id="rId9"/>
+    <sheet name="events{}" sheetId="27" r:id="rId10"/>
+    <sheet name="LCevents" sheetId="28" r:id="rId11"/>
+    <sheet name="act hooks{}" sheetId="26" r:id="rId12"/>
+    <sheet name="Middleware" sheetId="24" r:id="rId13"/>
+    <sheet name="act caching" sheetId="32" r:id="rId14"/>
+    <sheet name="settings{}depend()" sheetId="29" r:id="rId15"/>
+    <sheet name="ctx" sheetId="22" r:id="rId16"/>
+    <sheet name="Service (ES6)" sheetId="20" r:id="rId17"/>
+    <sheet name="API Gateway" sheetId="18" r:id="rId18"/>
+    <sheet name="Hooks" sheetId="38" r:id="rId19"/>
+    <sheet name="File up(down)load aliases" sheetId="35" r:id="rId20"/>
+    <sheet name="Response type" sheetId="36" r:id="rId21"/>
+    <sheet name="Authorization &amp; Authent" sheetId="37" r:id="rId22"/>
+    <sheet name="Transporter" sheetId="31" r:id="rId23"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -57,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1849" uniqueCount="1543">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="1607">
   <si>
     <t>Документация https://moleculer.services/docs/0.14/broker</t>
   </si>
@@ -18341,17 +18343,687 @@
   <si>
     <t>dotenv - https://www.npmjs.com/package/dotenv</t>
   </si>
+  <si>
+    <t>mkdir my-moleculer-project</t>
+  </si>
+  <si>
+    <t>cd my-moleculer-project</t>
+  </si>
+  <si>
+    <t>npm init -y</t>
+  </si>
+  <si>
+    <t>npm install nodemon eslint --save-dev</t>
+  </si>
+  <si>
+    <t>npm install moleculer moleculer-web --save</t>
+  </si>
+  <si>
+    <t>moleculer-web is the official Moleculer API gateway middleware to prpvision RESTful or WebSocket endpoints</t>
+  </si>
+  <si>
+    <t>Approach from book</t>
+  </si>
+  <si>
+    <t>my-molecular-project/
+│
+├── services/                    # Contains individual microservice definitions
+│   ├── users.service.js
+│   ├── orders.service.js
+│   └── payment.service.js
+│
+├── api/                         # API gateway configuration and routes
+│   └── api.service.js
+│
+├── bin/                         # Executable scripts, e.g., service launcher
+│   └── start.js
+│
+├── config/                      # Configuration files (environment, Molecular settings)
+│   ├── default.json
+│   ├── development.json
+│   └── production.json
+│
+├── test/                        # Unit and integration tests
+│   └── users.spec.js
+│
+├── .eslintrc.js                 # ESLint configuration
+├── .gitignore
+├── package.json
+└── README.md</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">"scripts": {
+    "start": "node bin/start.js",                    // Запуск приложения в production-режиме
+    "dev": "nodemon </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">--watch </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>services</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">--watch </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>api</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> --exec 'node bin/start.js'"   // Запуск в режиме разработки с автоперезагрузкой
+}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">dev — запуск с nodemon, который:
+1 Отслеживает изменения в папках </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>services</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> и </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>api</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (--watch)
+2 При обнаружении изменений автоматически перезапускает приложение (--exec)
+3 Удобно для разработки, не нужно перезапускать сервер вручную после каждого изменения кода</t>
+    </r>
+  </si>
+  <si>
+    <t>Simpler development</t>
+  </si>
+  <si>
+    <t>Local development with hot reloading</t>
+  </si>
+  <si>
+    <t>git</t>
+  </si>
+  <si>
+    <t>2. **Version Control Best Practices**: 
+   - Организуйте ветки по функционалу или микросервису, чтобы минимизировать сложные слияния.
+   - Исключите node_modules из репозитория через .gitignore для уменьшения размера репозитория.
+   - Вносите атомарные изменения, относящиеся к конкретным сервисам, чтобы упростить процесс ревью.</t>
+  </si>
+  <si>
+    <t>3. **Service Isolation and Testing**: 
+   - Отдельные сервисы могут тестироваться изолированно с помощью unit-тестов в директории test, которые помогают проверять интерфейсы перед интеграцией.
+   - Сфокусированные наборы тестов сокращают цикл обратной связи и повышают уверенность при развёртывании.</t>
+  </si>
+  <si>
+    <t>test/</t>
+  </si>
+  <si>
+    <t>bin/start.js</t>
+  </si>
+  <si>
+    <t>4. **Consistent Code Style**: 
+   - Используйте ESLint, интегрированный с IDE plugin and as a pre-commit Git хука, чтобы обеспечить единые стандарты кодирования среди всех контрибьюторов и предотвращать стилистические регрессии.</t>
+  </si>
+  <si>
+    <t>eslint</t>
+  </si>
+  <si>
+    <t>cicd</t>
+  </si>
+  <si>
+    <t>Typical steps
+- Installing dependencies through npm ci for reproducible installations
+- Running tests using frameworks such as Jest or Mocha, invoked via npm test
+- Performing linting checks with npm run lint
+- Deploying services using containerization or cloud frameworks, referencing environment-specific configuration files for dynamic setup</t>
+  </si>
+  <si>
+    <t>`https://habr.com/ru/companies/otus/articles/766774/</t>
+  </si>
+  <si>
+    <t>`https://t.me/Java_Iibrary/2477</t>
+  </si>
+  <si>
+    <t>проблемы с блокировкой потока</t>
+  </si>
+  <si>
+    <t>Пояснение! Когда пользователь отправляет запрос на сервер, при обычном сценарии этот запрос начинает бегать по всем серверу, а также другим серверам, возвращая ответ пользователю лишь в самый последний момент.
+Чтобы ускорить.
+1 Можно использовать Events, которые реализрованы в Moleculer js, тем самым возвращая в return action, к которому обратился пользователь готовый ответ, без ожидания, когда выполнят свою работу другие actions. Другие actions будут вызываны благодаря механизму подписки на Events
+2 Можно для REST использовать очереди задач для сложных запросов возвращая пользователю id job и периодически обновляя статус job. Appache Kafka, RabbitMQ...
+Можно использовать Graphql на фронте (схожий механизм с Socket), который может возвращать статус процесса.
+3 В java можно использовать CompletableFuture , который позволяет мгновенно вернуть ответ, который задействует HTTP поток для возвращения ответа без его ожидания</t>
+  </si>
+  <si>
+    <t>Moleculer предоставляет довольно уникальный инструмент для ускорения обработки пользовательских запросов на сервер. После получения запроса на один из обработчиков, ответ возвращается максимально быстро (без ожидания пользователем выполнения дополнительных работ другими сервисами и серверами). Дополнительные работы будут назначены, благодаря subscribtion механизму на Events в других actions</t>
+  </si>
+  <si>
+    <t>Event driven development (Аспектное программирование)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">смотри </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">2.3 Event-Driven Programming in MoleculerJS - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MoleculerJS EssentialsDefinitive Reference</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Services subscribe to events by defining event handlers in the events object. Handlers receive the event payload asynchronously, allowing non-blocking operations.
+Such patterns </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>mix event-driven</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>decoupling</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>the strict guarantees of request/response</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> workflows, balancing scalability and consistency.</t>
+    </r>
+  </si>
+  <si>
+    <t>mix event-driven decoupling +  the strict guarantees of request/response</t>
+  </si>
+  <si>
+    <t>Local Events</t>
+  </si>
+  <si>
+    <t>Global Events</t>
+  </si>
+  <si>
+    <t>Event Subscribers</t>
+  </si>
+  <si>
+    <t>Event Payload</t>
+  </si>
+  <si>
+    <t>Wildcard Subscriptions</t>
+  </si>
+  <si>
+    <t>Acknowledge Patterns</t>
+  </si>
+  <si>
+    <t>Workflow Orchestration</t>
+  </si>
+  <si>
+    <t>JSON-serializable data passed to handlers providing event context.</t>
+  </si>
+  <si>
+    <t>Combining events with actions or business transactions to ensure reliable processing.</t>
+  </si>
+  <si>
+    <t>Chaining event emissions and handlers to build scalable, reactive business processes.</t>
+  </si>
+  <si>
+    <t>Defined by the events object; can listen to specific or wildcard event names.</t>
+  </si>
+  <si>
+    <t>Use of * in event patterns to capture groups of events sharing prefixes or suffixes.</t>
+  </si>
+  <si>
+    <r>
+      <t>Emitted and consumed within a single service instance using </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>this.emit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Useful for decoupling internal logic.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Emitted on Molecular's event bus using </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ctx.emit </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>and handled by any subscriber across the network.</t>
+    </r>
+  </si>
+  <si>
+    <t>REST, JSON RPC, GraphQL</t>
+  </si>
+  <si>
+    <t>В REST вы создаете новый эндпоинт для каждой новой комбинации данных, потому что URL = ресурс.</t>
+  </si>
+  <si>
+    <t>Отличия</t>
+  </si>
+  <si>
+    <t>Json RPC</t>
+  </si>
+  <si>
+    <t>GraphQL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Преимущество! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>С Json RPC пример выше сократился бы до одного запроса</t>
+    </r>
+  </si>
+  <si>
+    <t>В JSON-RPC у вас один URL, а комбинации собираются на стороне клиента. Это экономит время разработки и делает API более гибким. Клиент диктует серверу, какие данные ему нужны и в какой комбинации</t>
+  </si>
+  <si>
+    <t>Добавление нового поля = клиент просто начинает его запрашивать. Сервер — "шведский стол" (бери что хочешь в любой комбинации)</t>
+  </si>
+  <si>
+    <t>[
+  {
+    "jsonrpc": "2.0",
+    "method": "getUser",
+    "params": [123],
+    "id": 1
+  },
+  {
+    "jsonrpc": "2.0",
+    "method": "getOrders",
+    "params": [123, {"limit": 5}],
+    "id": 2
+  },
+  {
+    "jsonrpc": "2.0",
+    "method": "calculateTax",
+    "params": [123, "2026-07"],
+    "id": 3
+  },
+  {
+    "jsonrpc": "2.0",
+    "method": "getUnreadNotifications",
+    "params": [123],
+    "id": 4
+  }
+]</t>
+  </si>
+  <si>
+    <t>[
+  {
+    "jsonrpc": "2.0",
+    "result": { "id": 123, "name": "Алексей" },
+    "id": 1
+  },
+  {
+    "jsonrpc": "2.0",
+    "result": [
+      { "id": 1, "sum": 1500 },
+      { "id": 2, "sum": 2300 }
+    ],
+    "id": 2
+  },
+  {
+    "jsonrpc": "2.0",
+    "result": 450.50,
+    "id": 3
+  },
+  {
+    "jsonrpc": "2.0",
+    "error": { "code": -32000, "message": "Service unavailable" },
+    "id": 4
+  }
+]</t>
+  </si>
+  <si>
+    <t>Запрос</t>
+  </si>
+  <si>
+    <t>Ответ</t>
+  </si>
+  <si>
+    <t>query {
+  user(id: 123) {
+    name
+    email
+  }
+  orders(userId: 123, limit: 5) {
+    id
+    sum
+  }
+  tax(userId: 123, month: "2026-07")
+  unreadNotifications(userId: 123)
+}</t>
+  </si>
+  <si>
+    <t>{
+  "data": {
+    "user": { "name": "Алексей", "email": "alex@mail.com" },
+    "orders": [ { "id": 1, "sum": 1500 } ],
+    "tax": 450.50,
+    "unreadNotifications": null
+  },
+  "errors": [
+    { "message": "Service unavailable", "path": ["unreadNotifications"] }
+  ]
+}</t>
+  </si>
+  <si>
+    <t>GraphQL делает то же самое, но в более структурированном виде. Вместо массива методов вы отправляете один запрос, описывающий структуру нужных данных</t>
+  </si>
+  <si>
+    <t>Сервер получает этот массив, параллельно (или последовательно) выполняет все 4 метода и возвращает</t>
+  </si>
+  <si>
+    <t>Вы отправляете один POST-запрос на URL /api/rpc, внутри которого массив из 4 вызовов</t>
+  </si>
+  <si>
+    <t>dotenv</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">// bin/start.js
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">require('dotenv').config(); </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                         // Загружаем переменные окружения из .env файла
+const { ServiceBroker } = require('moleculer');      // Импортируем класс ServiceBroker из библиотеки Moleculer
+const broker = new ServiceBroker({                  // Создаём экземпляр брокера с конфигурацией
+  nodeID: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>process.env.NODE_ID</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> || "node-1",          // Уникальный идентификатор узла (берётся из env, по умолчанию "node-1")
+  transporter: "NATS",                              // Транспорт для обмена сообщениями между сервисами (NATS)
+  logger: console,                                  // Логгер (вывод в консоль)
+  logLevel: "info"                                  // Уровень логирования (info, debug, error и т.д.)
+});
+broker.loadServices("./services");                  // Загружаем все сервисы из папки ./services
+broker.start();                                     // Запускаем брокер (стартуем все сервисы и подключаемся к транспорту)</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="48">
+  <fonts count="49">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -19043,7 +19715,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -19054,23 +19726,23 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -19088,7 +19760,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19106,7 +19778,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19127,7 +19799,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19148,7 +19820,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19166,10 +19838,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19178,28 +19850,28 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19208,49 +19880,49 @@
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="32" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19259,7 +19931,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19268,7 +19940,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19280,7 +19952,7 @@
     <xf numFmtId="49" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19289,22 +19961,22 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19316,89 +19988,92 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="29" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -19406,28 +20081,28 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="30" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="31" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -19437,6 +20112,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -19460,23 +20142,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>56028</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>84588</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>158754</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>127074</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>3161339</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>2285999</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1697430</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>820157</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="4" name="Рисунок 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{690A2FD4-172F-47B4-B487-4D18E80C53F3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47E8B52A-F659-460F-9AFF-066F11BCFD02}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -19492,8 +20174,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5990663" y="4091812"/>
-          <a:ext cx="3105311" cy="2201411"/>
+          <a:off x="2624048" y="18493515"/>
+          <a:ext cx="1548201" cy="677843"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -20629,16 +21311,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BE2ADE5-9A6F-4274-9C48-F960B495367E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{613720B3-4EFD-476A-A511-3737CA8EDAAD}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V27"/>
+  <dimension ref="A2:V6"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
     <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="105.21875" style="4" customWidth="1"/>
     <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
     <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
@@ -20685,238 +21367,1126 @@
       <c r="U2" s="5"/>
     </row>
     <row r="3" spans="1:22">
-      <c r="A3" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="C3" s="46" t="s">
-        <v>347</v>
-      </c>
+      <c r="C3" s="46"/>
       <c r="P3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="2"/>
     </row>
     <row r="4" spans="1:22">
-      <c r="A4" s="45" t="s">
-        <v>364</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="P4" s="1"/>
-      <c r="U4" s="1"/>
-      <c r="V4" s="2"/>
-    </row>
-    <row r="5" spans="1:22" ht="43.2">
-      <c r="A5" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="P5" s="1"/>
-      <c r="U5" s="1"/>
-      <c r="V5" s="2"/>
-    </row>
-    <row r="6" spans="1:22" ht="115.2">
-      <c r="A6" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="B6" s="48" t="s">
-        <v>367</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="P6" s="1"/>
-      <c r="U6" s="1"/>
-      <c r="V6" s="2"/>
-    </row>
-    <row r="7" spans="1:22" ht="57.6">
-      <c r="A7" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="P7" s="1"/>
-      <c r="U7" s="1"/>
-      <c r="V7" s="2"/>
-    </row>
-    <row r="8" spans="1:22" ht="28.8">
-      <c r="A8" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="C8" s="51" t="s">
-        <v>385</v>
-      </c>
-      <c r="P8" s="1"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="2"/>
-    </row>
-    <row r="9" spans="1:22">
-      <c r="A9" s="12" t="s">
-        <v>393</v>
-      </c>
-      <c r="C9" s="51"/>
-      <c r="P9" s="1"/>
-      <c r="U9" s="1"/>
-      <c r="V9" s="2"/>
-    </row>
-    <row r="10" spans="1:22" ht="187.2">
-      <c r="B10" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="C10" s="51"/>
-      <c r="P10" s="1"/>
-      <c r="U10" s="1"/>
-      <c r="V10" s="2"/>
-    </row>
-    <row r="11" spans="1:22" ht="28.8">
-      <c r="A11" s="45" t="s">
-        <v>1176</v>
-      </c>
-    </row>
-    <row r="12" spans="1:22">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2" t="s">
-        <v>580</v>
-      </c>
-      <c r="C12" s="95" t="s">
-        <v>1171</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22" ht="28.8">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2" t="s">
-        <v>581</v>
-      </c>
-      <c r="C13" s="95" t="s">
-        <v>1172</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2" t="s">
-        <v>582</v>
-      </c>
-      <c r="C14" s="95" t="s">
-        <v>1173</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" ht="72">
-      <c r="A15" s="2"/>
-      <c r="B15" s="1"/>
+      <c r="A4" s="12" t="s">
+        <v>1566</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="331.2">
+      <c r="B5" s="2" t="s">
+        <v>1567</v>
+      </c>
+      <c r="C5" s="133" t="s">
+        <v>1564</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22">
+      <c r="C6" s="133" t="s">
+        <v>1565</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03D965FF-3469-4ADC-BFBB-2C499831567E}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.39997558519241921"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V38"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="72.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3" s="97" t="s">
+        <v>896</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22" s="7" customFormat="1" ht="28.8">
+      <c r="A4" s="12" t="s">
+        <v>895</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="8"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="1"/>
+    </row>
+    <row r="5" spans="1:22" s="7" customFormat="1" ht="28.8">
+      <c r="A5" s="1"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="51" t="s">
+        <v>387</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="1"/>
+    </row>
+    <row r="6" spans="1:22" s="7" customFormat="1" ht="28.8">
+      <c r="A6" s="1"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="51" t="s">
+        <v>388</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="1"/>
+    </row>
+    <row r="7" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A7" s="1"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="51" t="s">
+        <v>389</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="1"/>
+    </row>
+    <row r="8" spans="1:22" s="7" customFormat="1" ht="28.8">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="42" t="s">
+        <v>337</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="1"/>
+    </row>
+    <row r="9" spans="1:22" s="7" customFormat="1" ht="216">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="52" t="s">
+        <v>427</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="1"/>
+    </row>
+    <row r="10" spans="1:22" s="7" customFormat="1">
+      <c r="A10" s="12" t="s">
+        <v>344</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="1"/>
+    </row>
+    <row r="11" spans="1:22" s="7" customFormat="1">
+      <c r="A11" s="49" t="s">
+        <v>1073</v>
+      </c>
+      <c r="B11" s="95"/>
+      <c r="C11" s="95"/>
+      <c r="D11" s="95"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="1"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="1"/>
+    </row>
+    <row r="12" spans="1:22" s="7" customFormat="1">
+      <c r="A12" s="95"/>
+      <c r="B12" s="95" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D12" s="95"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="1"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="1"/>
+    </row>
+    <row r="13" spans="1:22" s="7" customFormat="1">
+      <c r="A13" s="95"/>
+      <c r="B13" s="95" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>1078</v>
+      </c>
+      <c r="D13" s="95"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="1"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="2"/>
+      <c r="V13" s="1"/>
+    </row>
+    <row r="14" spans="1:22" s="7" customFormat="1">
+      <c r="A14" s="95"/>
+      <c r="B14" s="95" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D14" s="95"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="1"/>
+    </row>
+    <row r="15" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A15" s="95"/>
+      <c r="B15" s="95" t="s">
+        <v>1074</v>
+      </c>
       <c r="C15" s="2" t="s">
-        <v>1175</v>
-      </c>
-    </row>
-    <row r="16" spans="1:22" ht="43.2">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2" t="s">
-        <v>583</v>
-      </c>
-      <c r="C16" s="95" t="s">
-        <v>1174</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="12" t="s">
-        <v>1160</v>
-      </c>
-      <c r="C17" s="95"/>
-    </row>
-    <row r="18" spans="1:4" ht="57.6">
-      <c r="A18" s="2" t="s">
-        <v>1161</v>
-      </c>
-      <c r="C18" s="111" t="s">
-        <v>1179</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="72">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2" t="s">
-        <v>1169</v>
-      </c>
-      <c r="C19" s="95" t="s">
-        <v>1166</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="72">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2" t="s">
-        <v>1168</v>
+        <v>1075</v>
+      </c>
+      <c r="D15" s="95"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="8"/>
+      <c r="U15" s="2"/>
+      <c r="V15" s="1"/>
+    </row>
+    <row r="16" spans="1:22" s="7" customFormat="1">
+      <c r="A16" s="98" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B16" s="90"/>
+      <c r="C16" s="90"/>
+      <c r="D16" s="90"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="8"/>
+      <c r="U16" s="2"/>
+      <c r="V16" s="1"/>
+    </row>
+    <row r="17" spans="1:22" s="7" customFormat="1" ht="360">
+      <c r="A17" s="2" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B17" s="95" t="s">
+        <v>446</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D17" s="95" t="s">
+        <v>1072</v>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="8"/>
+      <c r="U17" s="2"/>
+      <c r="V17" s="1"/>
+    </row>
+    <row r="18" spans="1:22" s="7" customFormat="1" ht="288">
+      <c r="A18" s="52" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C18" s="59" t="s">
+        <v>1133</v>
+      </c>
+      <c r="D18" s="59" t="s">
+        <v>1134</v>
+      </c>
+      <c r="F18" s="1"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="1"/>
+      <c r="T18" s="8"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="1"/>
+    </row>
+    <row r="19" spans="1:22" s="7" customFormat="1">
+      <c r="A19" s="13" t="s">
+        <v>435</v>
+      </c>
+      <c r="B19" s="95"/>
+      <c r="C19" s="95"/>
+      <c r="D19" s="95"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="8"/>
+      <c r="U19" s="2"/>
+      <c r="V19" s="1"/>
+    </row>
+    <row r="20" spans="1:22" s="7" customFormat="1" ht="409.6">
+      <c r="A20" s="1"/>
+      <c r="B20" s="95" t="s">
+        <v>887</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1167</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="100.8">
-      <c r="A21" s="2" t="s">
-        <v>1170</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>1281</v>
-      </c>
-      <c r="C21" s="111" t="s">
-        <v>1180</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>1280</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="43.2">
-      <c r="A22" s="95" t="s">
-        <v>1159</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>831</v>
-      </c>
-      <c r="C22" s="95" t="s">
-        <v>1163</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>1165</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="43.2">
-      <c r="B23" s="95" t="s">
-        <v>1162</v>
-      </c>
-      <c r="C23" s="95" t="s">
-        <v>1164</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>1165</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="95"/>
-      <c r="B24" s="2" t="s">
-        <v>939</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>1165</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="95" t="s">
-        <v>391</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="D27" s="4"/>
+        <v>888</v>
+      </c>
+      <c r="D20" s="42" t="s">
+        <v>346</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="8"/>
+      <c r="U20" s="2"/>
+      <c r="V20" s="1"/>
+    </row>
+    <row r="21" spans="1:22" s="7" customFormat="1">
+      <c r="A21" s="44" t="s">
+        <v>428</v>
+      </c>
+      <c r="B21" s="59"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="1"/>
+      <c r="T21" s="8"/>
+      <c r="U21" s="2"/>
+      <c r="V21" s="1"/>
+    </row>
+    <row r="22" spans="1:22" s="7" customFormat="1" ht="28.8">
+      <c r="A22" s="2"/>
+      <c r="B22" s="42" t="s">
+        <v>340</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2"/>
+      <c r="S22" s="1"/>
+      <c r="T22" s="8"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="1"/>
+    </row>
+    <row r="23" spans="1:22" s="7" customFormat="1" ht="216">
+      <c r="A23" s="2" t="s">
+        <v>1084</v>
+      </c>
+      <c r="B23" s="52" t="s">
+        <v>430</v>
+      </c>
+      <c r="C23" s="52" t="s">
+        <v>429</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="8"/>
+      <c r="U23" s="2"/>
+      <c r="V23" s="1"/>
+    </row>
+    <row r="24" spans="1:22" s="7" customFormat="1" ht="72">
+      <c r="A24" s="2" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B24" s="52"/>
+      <c r="C24" s="95" t="s">
+        <v>1082</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="1"/>
+      <c r="T24" s="8"/>
+      <c r="U24" s="2"/>
+      <c r="V24" s="1"/>
+    </row>
+    <row r="25" spans="1:22" s="7" customFormat="1">
+      <c r="A25" s="12" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B25" s="45"/>
+      <c r="C25" s="105"/>
+      <c r="D25" s="12"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="1"/>
+      <c r="T25" s="8"/>
+      <c r="U25" s="2"/>
+      <c r="V25" s="1"/>
+    </row>
+    <row r="26" spans="1:22" s="7" customFormat="1" ht="72">
+      <c r="A26" s="129" t="s">
+        <v>1531</v>
+      </c>
+      <c r="B26" s="43" t="s">
+        <v>1523</v>
+      </c>
+      <c r="C26" s="43" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D26" s="43"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="P26" s="2"/>
+      <c r="Q26" s="2"/>
+      <c r="R26" s="2"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="8"/>
+      <c r="U26" s="2"/>
+      <c r="V26" s="1"/>
+    </row>
+    <row r="27" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A27" s="126" t="s">
+        <v>431</v>
+      </c>
+      <c r="B27" s="43" t="s">
+        <v>1521</v>
+      </c>
+      <c r="C27" s="127" t="s">
+        <v>1527</v>
+      </c>
+      <c r="D27" s="96" t="s">
+        <v>889</v>
+      </c>
+      <c r="F27" s="1"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="P27" s="2"/>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
+      <c r="S27" s="1"/>
+      <c r="T27" s="8"/>
+      <c r="U27" s="2"/>
+      <c r="V27" s="1"/>
+    </row>
+    <row r="28" spans="1:22" s="7" customFormat="1" ht="409.6">
+      <c r="A28" s="43"/>
+      <c r="B28" s="128" t="s">
+        <v>1530</v>
+      </c>
+      <c r="C28" s="125" t="s">
+        <v>1529</v>
+      </c>
+      <c r="D28" s="43"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="P28" s="2"/>
+      <c r="Q28" s="2"/>
+      <c r="R28" s="2"/>
+      <c r="S28" s="1"/>
+      <c r="T28" s="8"/>
+      <c r="U28" s="2"/>
+      <c r="V28" s="1"/>
+    </row>
+    <row r="29" spans="1:22" s="7" customFormat="1" ht="187.2">
+      <c r="A29" s="95"/>
+      <c r="B29" s="125" t="s">
+        <v>342</v>
+      </c>
+      <c r="C29" s="125" t="s">
+        <v>1524</v>
+      </c>
+      <c r="D29" s="95" t="s">
+        <v>890</v>
+      </c>
+      <c r="F29" s="1"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="P29" s="2"/>
+      <c r="Q29" s="2"/>
+      <c r="R29" s="2"/>
+      <c r="S29" s="1"/>
+      <c r="T29" s="8"/>
+      <c r="U29" s="2"/>
+      <c r="V29" s="1"/>
+    </row>
+    <row r="30" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A30" s="126" t="s">
+        <v>432</v>
+      </c>
+      <c r="B30" s="43" t="s">
+        <v>893</v>
+      </c>
+      <c r="C30" s="127" t="s">
+        <v>1526</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="P30" s="2"/>
+      <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="8"/>
+      <c r="U30" s="2"/>
+      <c r="V30" s="1"/>
+    </row>
+    <row r="31" spans="1:22" s="7" customFormat="1" ht="201.6">
+      <c r="A31" s="106"/>
+      <c r="B31" s="95" t="s">
+        <v>894</v>
+      </c>
+      <c r="C31" s="125" t="s">
+        <v>1525</v>
+      </c>
+      <c r="D31" s="43" t="s">
+        <v>891</v>
+      </c>
+      <c r="F31" s="1"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="P31" s="2"/>
+      <c r="Q31" s="2"/>
+      <c r="R31" s="2"/>
+      <c r="S31" s="1"/>
+      <c r="T31" s="8"/>
+      <c r="U31" s="2"/>
+      <c r="V31" s="1"/>
+    </row>
+    <row r="32" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A32" s="126" t="s">
+        <v>434</v>
+      </c>
+      <c r="B32" s="43" t="s">
+        <v>892</v>
+      </c>
+      <c r="C32" s="127" t="s">
+        <v>1528</v>
+      </c>
+      <c r="D32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="P32" s="2"/>
+      <c r="Q32" s="2"/>
+      <c r="R32" s="2"/>
+      <c r="S32" s="1"/>
+      <c r="T32" s="8"/>
+      <c r="U32" s="2"/>
+      <c r="V32" s="1"/>
+    </row>
+    <row r="33" spans="1:22" s="7" customFormat="1" ht="72">
+      <c r="A33" s="52"/>
+      <c r="B33" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="C33" s="125" t="s">
+        <v>433</v>
+      </c>
+      <c r="D33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="P33" s="2"/>
+      <c r="Q33" s="2"/>
+      <c r="R33" s="2"/>
+      <c r="S33" s="1"/>
+      <c r="T33" s="8"/>
+      <c r="U33" s="2"/>
+      <c r="V33" s="1"/>
+    </row>
+    <row r="34" spans="1:22">
+      <c r="A34" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22">
+      <c r="A35" s="1" t="s">
+        <v>1112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" ht="187.2">
+      <c r="C36" s="95" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22">
+      <c r="A37" s="1" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" ht="158.4">
+      <c r="C38" s="95" t="s">
+        <v>1114</v>
+      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D88F61F-8C7C-4710-8F38-D46F66310E17}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.39997558519241921"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V10"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="72.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3" s="97" t="s">
+        <v>897</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22" s="7" customFormat="1">
+      <c r="A4" s="12" t="s">
+        <v>448</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="8"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="1"/>
+    </row>
+    <row r="5" spans="1:22" ht="360">
+      <c r="C5" s="52" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="374.4">
+      <c r="A6" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="C6" s="68" t="s">
+        <v>791</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" s="7" customFormat="1" ht="172.8">
+      <c r="A7" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>787</v>
+      </c>
+      <c r="C7" s="68" t="s">
+        <v>783</v>
+      </c>
+      <c r="D7" s="68" t="s">
+        <v>786</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="1"/>
+    </row>
+    <row r="8" spans="1:22" s="7" customFormat="1" ht="409.6">
+      <c r="A8" s="90"/>
+      <c r="B8" s="93" t="s">
+        <v>870</v>
+      </c>
+      <c r="C8" s="93" t="s">
+        <v>869</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="1"/>
+    </row>
+    <row r="9" spans="1:22" s="7" customFormat="1" ht="187.2">
+      <c r="A9" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="C9" s="68" t="s">
+        <v>784</v>
+      </c>
+      <c r="D9" s="68" t="s">
+        <v>785</v>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="1"/>
+    </row>
+    <row r="10" spans="1:22" s="7" customFormat="1" ht="172.8">
+      <c r="A10" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>789</v>
+      </c>
+      <c r="C10" s="68" t="s">
+        <v>782</v>
+      </c>
+      <c r="D10" s="68" t="s">
+        <v>781</v>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7C45E35-A0E9-4FBE-88F3-CE4B282CF0DD}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -22071,7 +23641,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F722A6B-FDD4-4F28-A73E-E1B84FE9A13E}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -22835,7 +24405,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2EDDD90-7CFC-46CE-93A4-19D76FB6A77B}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -23263,7 +24833,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF050F64-E219-48FB-BA24-6D9B0B37599F}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -23604,7 +25174,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9400A441-6B67-47CF-87A5-3C3813CBCD51}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -23984,7 +25554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C7DACD-972C-4F9B-8B6E-158B3A84F36B}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -24100,7 +25670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84D070D-9F43-498E-8C8B-DA56F9B43AEF}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -26190,13 +27760,13 @@
       <c r="V87" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="22" type="noConversion"/>
+  <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{215A08A6-8FA5-47FE-AD3E-099EDF44B417}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -26502,7 +28072,276 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BE2ADE5-9A6F-4274-9C48-F960B495367E}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3" s="46" t="s">
+        <v>347</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22">
+      <c r="A4" s="45" t="s">
+        <v>364</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="P4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="2"/>
+    </row>
+    <row r="5" spans="1:22" ht="43.2">
+      <c r="A5" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="P5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="2"/>
+    </row>
+    <row r="6" spans="1:22" ht="115.2">
+      <c r="A6" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>367</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="P6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="2"/>
+    </row>
+    <row r="7" spans="1:22" ht="57.6">
+      <c r="A7" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="P7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="2"/>
+    </row>
+    <row r="8" spans="1:22" ht="28.8">
+      <c r="A8" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="C8" s="51" t="s">
+        <v>385</v>
+      </c>
+      <c r="P8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="2"/>
+    </row>
+    <row r="9" spans="1:22" ht="28.8">
+      <c r="A9" s="45" t="s">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="C10" s="95" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="28.8">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="C11" s="95" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="C12" s="95" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="72">
+      <c r="A13" s="2"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="2" t="s">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="43.2">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="C14" s="95" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22">
+      <c r="A15" s="12" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C15" s="95"/>
+    </row>
+    <row r="16" spans="1:22" ht="57.6">
+      <c r="A16" s="2" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C16" s="111" t="s">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="72">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C17" s="95" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="72">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2" t="s">
+        <v>1168</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="100.8">
+      <c r="A19" s="2" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>1281</v>
+      </c>
+      <c r="C19" s="111" t="s">
+        <v>1180</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>1280</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="43.2">
+      <c r="A20" s="95" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>831</v>
+      </c>
+      <c r="C20" s="95" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="43.2">
+      <c r="B21" s="95" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C21" s="95" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="95"/>
+      <c r="B22" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="95" t="s">
+        <v>391</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="D25" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="23" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E63D7CF-A8C1-4EE2-B24F-BB6423312324}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -26644,7 +28483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0E1A7F4-4156-43BA-A471-45FED5CB2B12}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -26792,122 +28631,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11C0BAE5-4B5A-4ED9-9078-DE65AE578F59}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A2:V9"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" style="8"/>
-    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.77734375" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:22">
-      <c r="A2" s="3"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="U2" s="5"/>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="C3" s="46" t="s">
-        <v>373</v>
-      </c>
-      <c r="P3" s="1"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:22">
-      <c r="A4" s="50" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22">
-      <c r="A5" s="1" t="s">
-        <v>375</v>
-      </c>
-      <c r="C5" s="48" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22">
-      <c r="A6" s="1" t="s">
-        <v>378</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="C6" s="48" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22">
-      <c r="A7" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="C7" s="48" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22">
-      <c r="A8" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="C8" s="48" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22" ht="28.8">
-      <c r="C9" s="48" t="s">
-        <v>384</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC0D01A-891F-4564-985B-BABA4F41741B}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -27041,7 +28765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C83401B-1940-4C7B-967F-92D40F8BF33D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -27248,6 +28972,594 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11C0BAE5-4B5A-4ED9-9078-DE65AE578F59}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V16"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="C3" s="46" t="s">
+        <v>373</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22">
+      <c r="A4" s="50" t="s">
+        <v>374</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22">
+      <c r="A5" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22">
+      <c r="A6" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22">
+      <c r="A7" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22">
+      <c r="A8" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="28.8">
+      <c r="C9" s="48" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22">
+      <c r="A11" s="50" t="s">
+        <v>1549</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22">
+      <c r="A12" s="1" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
+      <c r="A13" s="1" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22">
+      <c r="A14" s="1" t="s">
+        <v>1545</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="28.8">
+      <c r="A15" s="1" t="s">
+        <v>1547</v>
+      </c>
+      <c r="C15" s="133" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22">
+      <c r="A16" s="1" t="s">
+        <v>1546</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA45549C-F4E3-4DE8-8796-B64020ED8004}">
+  <sheetPr>
+    <tabColor rgb="FF7030A0"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V42"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="105.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3" s="46" t="s">
+        <v>347</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22">
+      <c r="A4" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="C4" s="51"/>
+      <c r="P4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="2"/>
+    </row>
+    <row r="5" spans="1:22" ht="360">
+      <c r="B5" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>1550</v>
+      </c>
+      <c r="P5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="2"/>
+    </row>
+    <row r="6" spans="1:22">
+      <c r="A6" s="12" t="s">
+        <v>1559</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" s="7" customFormat="1" ht="244.8">
+      <c r="A7" s="1" t="s">
+        <v>1605</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="C7" s="133" t="s">
+        <v>1606</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="1"/>
+    </row>
+    <row r="8" spans="1:22">
+      <c r="A8" s="3"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="U8" s="5"/>
+    </row>
+    <row r="9" spans="1:22" s="90" customFormat="1">
+      <c r="B9" s="59"/>
+      <c r="C9" s="135" t="s">
+        <v>1553</v>
+      </c>
+      <c r="G9" s="59"/>
+      <c r="P9" s="59"/>
+      <c r="Q9" s="59"/>
+      <c r="R9" s="59"/>
+      <c r="S9" s="59"/>
+      <c r="T9" s="134"/>
+      <c r="U9" s="59"/>
+    </row>
+    <row r="10" spans="1:22">
+      <c r="A10" s="12" t="s">
+        <v>1533</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="115.2">
+      <c r="A11" s="1" t="s">
+        <v>1554</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>1552</v>
+      </c>
+      <c r="C11" s="133" t="s">
+        <v>1551</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22">
+      <c r="A12" s="12" t="s">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="57.6">
+      <c r="C13" s="133" t="s">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22">
+      <c r="A14" s="12" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="57.6">
+      <c r="C15" s="133" t="s">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22">
+      <c r="A16" s="12" t="s">
+        <v>1561</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" ht="43.2">
+      <c r="C17" s="133" t="s">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21">
+      <c r="A18" s="12" t="s">
+        <v>1562</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" ht="86.4">
+      <c r="C19" s="133" t="s">
+        <v>1563</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21">
+      <c r="A20" s="3"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="5"/>
+      <c r="S20" s="5"/>
+      <c r="U20" s="5"/>
+    </row>
+    <row r="21" spans="1:21" s="90" customFormat="1">
+      <c r="B21" s="59"/>
+      <c r="C21" s="135" t="s">
+        <v>1569</v>
+      </c>
+      <c r="G21" s="59"/>
+      <c r="P21" s="59"/>
+      <c r="Q21" s="59"/>
+      <c r="R21" s="59"/>
+      <c r="S21" s="59"/>
+      <c r="T21" s="134"/>
+      <c r="U21" s="59"/>
+    </row>
+    <row r="22" spans="1:21" ht="57.6">
+      <c r="C22" s="133" t="s">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" ht="57.6">
+      <c r="A23" s="133" t="s">
+        <v>1572</v>
+      </c>
+      <c r="C23" s="133" t="s">
+        <v>1571</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>1570</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21">
+      <c r="A24" s="12" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21">
+      <c r="A25" s="1" t="s">
+        <v>1573</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>1585</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21">
+      <c r="A26" s="1" t="s">
+        <v>1574</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21">
+      <c r="A27" s="1" t="s">
+        <v>1575</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>1583</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21">
+      <c r="A28" s="1" t="s">
+        <v>1576</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21">
+      <c r="A29" s="1" t="s">
+        <v>1577</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>1584</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21">
+      <c r="A30" s="1" t="s">
+        <v>1578</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21">
+      <c r="A31" s="1" t="s">
+        <v>1579</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>1582</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21">
+      <c r="A33" s="3"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="P33" s="5"/>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="U33" s="5"/>
+    </row>
+    <row r="34" spans="1:21" s="90" customFormat="1">
+      <c r="B34" s="59"/>
+      <c r="C34" s="135" t="s">
+        <v>1587</v>
+      </c>
+      <c r="G34" s="59"/>
+      <c r="P34" s="59"/>
+      <c r="Q34" s="59"/>
+      <c r="R34" s="59"/>
+      <c r="S34" s="59"/>
+      <c r="T34" s="134"/>
+      <c r="U34" s="59"/>
+    </row>
+    <row r="35" spans="1:21">
+      <c r="A35" s="12" t="s">
+        <v>1589</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" ht="72">
+      <c r="A36" s="1" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>1592</v>
+      </c>
+      <c r="C36" s="133" t="s">
+        <v>1588</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" ht="28.8">
+      <c r="A37" s="1" t="s">
+        <v>1590</v>
+      </c>
+      <c r="B37" s="133" t="s">
+        <v>1593</v>
+      </c>
+      <c r="C37" s="133" t="s">
+        <v>1594</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" ht="28.8">
+      <c r="A38" s="1" t="s">
+        <v>1591</v>
+      </c>
+      <c r="C38" s="133" t="s">
+        <v>1595</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21">
+      <c r="A39" s="12" t="s">
+        <v>1590</v>
+      </c>
+      <c r="B39" s="45" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C39" s="136" t="s">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" ht="374.4">
+      <c r="A40" s="133" t="s">
+        <v>1604</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>1596</v>
+      </c>
+      <c r="C40" s="133" t="s">
+        <v>1597</v>
+      </c>
+      <c r="D40" s="133" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21">
+      <c r="A41" s="12" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B41" s="45"/>
+      <c r="C41" s="60"/>
+    </row>
+    <row r="42" spans="1:21" ht="172.8">
+      <c r="A42" s="2" t="s">
+        <v>1602</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>1600</v>
+      </c>
+      <c r="C42" s="133" t="s">
+        <v>1601</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC501503-0164-402D-9D9C-86B5F52AE94D}">
   <sheetPr>
     <tabColor theme="1"/>
@@ -28072,7 +30384,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{948CE0B5-C565-4729-8A1A-36CD87669389}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -28745,7 +31057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53293E74-C56C-43CE-8332-3FF6CCF78D58}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -30835,7 +33147,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47DCDB03-35F5-4E59-94D1-F4F42160A968}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -32916,7 +35228,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{488D8CBB-84D5-4AB1-A098-C4B0F9061CFB}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -33638,1094 +35950,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03D965FF-3469-4ADC-BFBB-2C499831567E}">
-  <sheetPr>
-    <tabColor theme="5" tint="0.39997558519241921"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A2:V38"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="72.21875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" style="8"/>
-    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.77734375" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:22">
-      <c r="A2" s="3"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="U2" s="5"/>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="C3" s="97" t="s">
-        <v>896</v>
-      </c>
-      <c r="P3" s="1"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:22" s="7" customFormat="1" ht="28.8">
-      <c r="A4" s="12" t="s">
-        <v>895</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="1"/>
-      <c r="T4" s="8"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="1"/>
-    </row>
-    <row r="5" spans="1:22" s="7" customFormat="1" ht="28.8">
-      <c r="A5" s="1"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="51" t="s">
-        <v>387</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="1"/>
-    </row>
-    <row r="6" spans="1:22" s="7" customFormat="1" ht="28.8">
-      <c r="A6" s="1"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="51" t="s">
-        <v>388</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="8"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="1"/>
-    </row>
-    <row r="7" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="51" t="s">
-        <v>389</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="8"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="1"/>
-    </row>
-    <row r="8" spans="1:22" s="7" customFormat="1" ht="28.8">
-      <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="42" t="s">
-        <v>337</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="1"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="1"/>
-    </row>
-    <row r="9" spans="1:22" s="7" customFormat="1" ht="216">
-      <c r="A9" s="1"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="52" t="s">
-        <v>427</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="8"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="1"/>
-    </row>
-    <row r="10" spans="1:22" s="7" customFormat="1">
-      <c r="A10" s="12" t="s">
-        <v>344</v>
-      </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="1"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="1"/>
-    </row>
-    <row r="11" spans="1:22" s="7" customFormat="1">
-      <c r="A11" s="49" t="s">
-        <v>1073</v>
-      </c>
-      <c r="B11" s="95"/>
-      <c r="C11" s="95"/>
-      <c r="D11" s="95"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="1"/>
-      <c r="T11" s="8"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="1"/>
-    </row>
-    <row r="12" spans="1:22" s="7" customFormat="1">
-      <c r="A12" s="95"/>
-      <c r="B12" s="95" t="s">
-        <v>1081</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>1080</v>
-      </c>
-      <c r="D12" s="95"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="1"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="2"/>
-      <c r="V12" s="1"/>
-    </row>
-    <row r="13" spans="1:22" s="7" customFormat="1">
-      <c r="A13" s="95"/>
-      <c r="B13" s="95" t="s">
-        <v>1079</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>1078</v>
-      </c>
-      <c r="D13" s="95"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="1"/>
-    </row>
-    <row r="14" spans="1:22" s="7" customFormat="1">
-      <c r="A14" s="95"/>
-      <c r="B14" s="95" t="s">
-        <v>1077</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>1076</v>
-      </c>
-      <c r="D14" s="95"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="8"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="1"/>
-    </row>
-    <row r="15" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A15" s="95"/>
-      <c r="B15" s="95" t="s">
-        <v>1074</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>1075</v>
-      </c>
-      <c r="D15" s="95"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="1"/>
-      <c r="T15" s="8"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="1"/>
-    </row>
-    <row r="16" spans="1:22" s="7" customFormat="1">
-      <c r="A16" s="98" t="s">
-        <v>1132</v>
-      </c>
-      <c r="B16" s="90"/>
-      <c r="C16" s="90"/>
-      <c r="D16" s="90"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="8"/>
-      <c r="U16" s="2"/>
-      <c r="V16" s="1"/>
-    </row>
-    <row r="17" spans="1:22" s="7" customFormat="1" ht="360">
-      <c r="A17" s="2" t="s">
-        <v>1126</v>
-      </c>
-      <c r="B17" s="95" t="s">
-        <v>446</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>1071</v>
-      </c>
-      <c r="D17" s="95" t="s">
-        <v>1072</v>
-      </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="8"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="1"/>
-    </row>
-    <row r="18" spans="1:22" s="7" customFormat="1" ht="288">
-      <c r="A18" s="52" t="s">
-        <v>1127</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>1135</v>
-      </c>
-      <c r="C18" s="59" t="s">
-        <v>1133</v>
-      </c>
-      <c r="D18" s="59" t="s">
-        <v>1134</v>
-      </c>
-      <c r="F18" s="1"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="8"/>
-      <c r="U18" s="2"/>
-      <c r="V18" s="1"/>
-    </row>
-    <row r="19" spans="1:22" s="7" customFormat="1">
-      <c r="A19" s="13" t="s">
-        <v>435</v>
-      </c>
-      <c r="B19" s="95"/>
-      <c r="C19" s="95"/>
-      <c r="D19" s="95"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="8"/>
-      <c r="U19" s="2"/>
-      <c r="V19" s="1"/>
-    </row>
-    <row r="20" spans="1:22" s="7" customFormat="1" ht="409.6">
-      <c r="A20" s="1"/>
-      <c r="B20" s="95" t="s">
-        <v>887</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>888</v>
-      </c>
-      <c r="D20" s="42" t="s">
-        <v>346</v>
-      </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="8"/>
-      <c r="U20" s="2"/>
-      <c r="V20" s="1"/>
-    </row>
-    <row r="21" spans="1:22" s="7" customFormat="1">
-      <c r="A21" s="44" t="s">
-        <v>428</v>
-      </c>
-      <c r="B21" s="59"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="8"/>
-      <c r="U21" s="2"/>
-      <c r="V21" s="1"/>
-    </row>
-    <row r="22" spans="1:22" s="7" customFormat="1" ht="28.8">
-      <c r="A22" s="2"/>
-      <c r="B22" s="42" t="s">
-        <v>340</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D22" s="2"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="8"/>
-      <c r="U22" s="2"/>
-      <c r="V22" s="1"/>
-    </row>
-    <row r="23" spans="1:22" s="7" customFormat="1" ht="216">
-      <c r="A23" s="2" t="s">
-        <v>1084</v>
-      </c>
-      <c r="B23" s="52" t="s">
-        <v>430</v>
-      </c>
-      <c r="C23" s="52" t="s">
-        <v>429</v>
-      </c>
-      <c r="D23" s="2"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="8"/>
-      <c r="U23" s="2"/>
-      <c r="V23" s="1"/>
-    </row>
-    <row r="24" spans="1:22" s="7" customFormat="1" ht="72">
-      <c r="A24" s="2" t="s">
-        <v>1083</v>
-      </c>
-      <c r="B24" s="52"/>
-      <c r="C24" s="95" t="s">
-        <v>1082</v>
-      </c>
-      <c r="D24" s="2"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="1"/>
-      <c r="T24" s="8"/>
-      <c r="U24" s="2"/>
-      <c r="V24" s="1"/>
-    </row>
-    <row r="25" spans="1:22" s="7" customFormat="1">
-      <c r="A25" s="12" t="s">
-        <v>1085</v>
-      </c>
-      <c r="B25" s="45"/>
-      <c r="C25" s="105"/>
-      <c r="D25" s="12"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="8"/>
-      <c r="U25" s="2"/>
-      <c r="V25" s="1"/>
-    </row>
-    <row r="26" spans="1:22" s="7" customFormat="1" ht="72">
-      <c r="A26" s="129" t="s">
-        <v>1531</v>
-      </c>
-      <c r="B26" s="43" t="s">
-        <v>1523</v>
-      </c>
-      <c r="C26" s="43" t="s">
-        <v>1072</v>
-      </c>
-      <c r="D26" s="43"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
-      <c r="P26" s="2"/>
-      <c r="Q26" s="2"/>
-      <c r="R26" s="2"/>
-      <c r="S26" s="1"/>
-      <c r="T26" s="8"/>
-      <c r="U26" s="2"/>
-      <c r="V26" s="1"/>
-    </row>
-    <row r="27" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A27" s="126" t="s">
-        <v>431</v>
-      </c>
-      <c r="B27" s="43" t="s">
-        <v>1521</v>
-      </c>
-      <c r="C27" s="127" t="s">
-        <v>1527</v>
-      </c>
-      <c r="D27" s="96" t="s">
-        <v>889</v>
-      </c>
-      <c r="F27" s="1"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-      <c r="K27" s="1"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="P27" s="2"/>
-      <c r="Q27" s="2"/>
-      <c r="R27" s="2"/>
-      <c r="S27" s="1"/>
-      <c r="T27" s="8"/>
-      <c r="U27" s="2"/>
-      <c r="V27" s="1"/>
-    </row>
-    <row r="28" spans="1:22" s="7" customFormat="1" ht="409.6">
-      <c r="A28" s="43"/>
-      <c r="B28" s="128" t="s">
-        <v>1530</v>
-      </c>
-      <c r="C28" s="125" t="s">
-        <v>1529</v>
-      </c>
-      <c r="D28" s="43"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
-      <c r="P28" s="2"/>
-      <c r="Q28" s="2"/>
-      <c r="R28" s="2"/>
-      <c r="S28" s="1"/>
-      <c r="T28" s="8"/>
-      <c r="U28" s="2"/>
-      <c r="V28" s="1"/>
-    </row>
-    <row r="29" spans="1:22" s="7" customFormat="1" ht="187.2">
-      <c r="A29" s="95"/>
-      <c r="B29" s="125" t="s">
-        <v>342</v>
-      </c>
-      <c r="C29" s="125" t="s">
-        <v>1524</v>
-      </c>
-      <c r="D29" s="95" t="s">
-        <v>890</v>
-      </c>
-      <c r="F29" s="1"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="P29" s="2"/>
-      <c r="Q29" s="2"/>
-      <c r="R29" s="2"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="8"/>
-      <c r="U29" s="2"/>
-      <c r="V29" s="1"/>
-    </row>
-    <row r="30" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A30" s="126" t="s">
-        <v>432</v>
-      </c>
-      <c r="B30" s="43" t="s">
-        <v>893</v>
-      </c>
-      <c r="C30" s="127" t="s">
-        <v>1526</v>
-      </c>
-      <c r="D30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="1"/>
-      <c r="T30" s="8"/>
-      <c r="U30" s="2"/>
-      <c r="V30" s="1"/>
-    </row>
-    <row r="31" spans="1:22" s="7" customFormat="1" ht="201.6">
-      <c r="A31" s="106"/>
-      <c r="B31" s="95" t="s">
-        <v>894</v>
-      </c>
-      <c r="C31" s="125" t="s">
-        <v>1525</v>
-      </c>
-      <c r="D31" s="43" t="s">
-        <v>891</v>
-      </c>
-      <c r="F31" s="1"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="K31" s="1"/>
-      <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="P31" s="2"/>
-      <c r="Q31" s="2"/>
-      <c r="R31" s="2"/>
-      <c r="S31" s="1"/>
-      <c r="T31" s="8"/>
-      <c r="U31" s="2"/>
-      <c r="V31" s="1"/>
-    </row>
-    <row r="32" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A32" s="126" t="s">
-        <v>434</v>
-      </c>
-      <c r="B32" s="43" t="s">
-        <v>892</v>
-      </c>
-      <c r="C32" s="127" t="s">
-        <v>1528</v>
-      </c>
-      <c r="D32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="K32" s="1"/>
-      <c r="L32" s="1"/>
-      <c r="M32" s="1"/>
-      <c r="N32" s="1"/>
-      <c r="P32" s="2"/>
-      <c r="Q32" s="2"/>
-      <c r="R32" s="2"/>
-      <c r="S32" s="1"/>
-      <c r="T32" s="8"/>
-      <c r="U32" s="2"/>
-      <c r="V32" s="1"/>
-    </row>
-    <row r="33" spans="1:22" s="7" customFormat="1" ht="72">
-      <c r="A33" s="52"/>
-      <c r="B33" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="C33" s="125" t="s">
-        <v>433</v>
-      </c>
-      <c r="D33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="K33" s="1"/>
-      <c r="L33" s="1"/>
-      <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
-      <c r="P33" s="2"/>
-      <c r="Q33" s="2"/>
-      <c r="R33" s="2"/>
-      <c r="S33" s="1"/>
-      <c r="T33" s="8"/>
-      <c r="U33" s="2"/>
-      <c r="V33" s="1"/>
-    </row>
-    <row r="34" spans="1:22">
-      <c r="A34" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="35" spans="1:22">
-      <c r="A35" s="1" t="s">
-        <v>1112</v>
-      </c>
-    </row>
-    <row r="36" spans="1:22" ht="187.2">
-      <c r="C36" s="95" t="s">
-        <v>1115</v>
-      </c>
-    </row>
-    <row r="37" spans="1:22">
-      <c r="A37" s="1" t="s">
-        <v>1113</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22" ht="158.4">
-      <c r="C38" s="95" t="s">
-        <v>1114</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D88F61F-8C7C-4710-8F38-D46F66310E17}">
-  <sheetPr>
-    <tabColor theme="5" tint="0.39997558519241921"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A2:V10"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="72.21875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" style="8"/>
-    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.77734375" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:22">
-      <c r="A2" s="3"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="U2" s="5"/>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="C3" s="97" t="s">
-        <v>897</v>
-      </c>
-      <c r="P3" s="1"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:22" s="7" customFormat="1">
-      <c r="A4" s="12" t="s">
-        <v>448</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="1"/>
-      <c r="T4" s="8"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="1"/>
-    </row>
-    <row r="5" spans="1:22" ht="360">
-      <c r="C5" s="52" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22" ht="374.4">
-      <c r="A6" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C6" s="68" t="s">
-        <v>791</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22" s="7" customFormat="1" ht="172.8">
-      <c r="A7" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>787</v>
-      </c>
-      <c r="C7" s="68" t="s">
-        <v>783</v>
-      </c>
-      <c r="D7" s="68" t="s">
-        <v>786</v>
-      </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="8"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="1"/>
-    </row>
-    <row r="8" spans="1:22" s="7" customFormat="1" ht="409.6">
-      <c r="A8" s="90"/>
-      <c r="B8" s="93" t="s">
-        <v>870</v>
-      </c>
-      <c r="C8" s="93" t="s">
-        <v>869</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="1"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="1"/>
-    </row>
-    <row r="9" spans="1:22" s="7" customFormat="1" ht="187.2">
-      <c r="A9" s="1" t="s">
-        <v>453</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>788</v>
-      </c>
-      <c r="C9" s="68" t="s">
-        <v>784</v>
-      </c>
-      <c r="D9" s="68" t="s">
-        <v>785</v>
-      </c>
-      <c r="F9" s="1"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="8"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="1"/>
-    </row>
-    <row r="10" spans="1:22" s="7" customFormat="1" ht="172.8">
-      <c r="A10" s="1" t="s">
-        <v>454</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>789</v>
-      </c>
-      <c r="C10" s="68" t="s">
-        <v>782</v>
-      </c>
-      <c r="D10" s="68" t="s">
-        <v>781</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="1"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
save 22 07 2026
</commit_message>
<xml_diff>
--- a/4 четверть_10_JavaScript_MoleculerJS.xlsx
+++ b/4 четверть_10_JavaScript_MoleculerJS.xlsx
@@ -8,34 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC03B171-CC95-46F3-9DA5-2C45E5DAA4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A027E8-1EF1-4383-AB28-3AEEC3E254D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4470" yWindow="-18225" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-810" yWindow="-14745" windowWidth="23010" windowHeight="11130" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Для изучения" sheetId="40" r:id="rId1"/>
     <sheet name="Basics" sheetId="12" r:id="rId2"/>
-    <sheet name="init new proj" sheetId="15" r:id="rId3"/>
-    <sheet name="Proj architecture" sheetId="39" r:id="rId4"/>
-    <sheet name="MoleculerError (Controller)" sheetId="33" r:id="rId5"/>
-    <sheet name="SB, config.js, env, Logging" sheetId="19" r:id="rId6"/>
-    <sheet name="ServiceBroker" sheetId="13" r:id="rId7"/>
-    <sheet name="Service" sheetId="17" r:id="rId8"/>
-    <sheet name="mixins{}" sheetId="30" r:id="rId9"/>
-    <sheet name="events{}" sheetId="27" r:id="rId10"/>
-    <sheet name="LCevents" sheetId="28" r:id="rId11"/>
-    <sheet name="act hooks{}" sheetId="26" r:id="rId12"/>
-    <sheet name="Middleware" sheetId="24" r:id="rId13"/>
-    <sheet name="act caching" sheetId="32" r:id="rId14"/>
-    <sheet name="settings{}depend()" sheetId="29" r:id="rId15"/>
-    <sheet name="ctx" sheetId="22" r:id="rId16"/>
-    <sheet name="Service (ES6)" sheetId="20" r:id="rId17"/>
-    <sheet name="API Gateway" sheetId="18" r:id="rId18"/>
-    <sheet name="Hooks" sheetId="38" r:id="rId19"/>
-    <sheet name="File up(down)load aliases" sheetId="35" r:id="rId20"/>
-    <sheet name="Response type" sheetId="36" r:id="rId21"/>
-    <sheet name="Authorization &amp; Authent" sheetId="37" r:id="rId22"/>
-    <sheet name="Transporter" sheetId="31" r:id="rId23"/>
+    <sheet name="DB Adapters" sheetId="41" r:id="rId3"/>
+    <sheet name="init new proj" sheetId="15" r:id="rId4"/>
+    <sheet name="Proj architecture" sheetId="39" r:id="rId5"/>
+    <sheet name="MoleculerError (Controller)" sheetId="33" r:id="rId6"/>
+    <sheet name="SB, config.js, env, Logging" sheetId="19" r:id="rId7"/>
+    <sheet name="ServiceBroker" sheetId="13" r:id="rId8"/>
+    <sheet name="Service" sheetId="17" r:id="rId9"/>
+    <sheet name="mixins{}" sheetId="30" r:id="rId10"/>
+    <sheet name="events{}" sheetId="27" r:id="rId11"/>
+    <sheet name="LCevents" sheetId="28" r:id="rId12"/>
+    <sheet name="act hooks{}" sheetId="26" r:id="rId13"/>
+    <sheet name="Middleware" sheetId="24" r:id="rId14"/>
+    <sheet name="act caching" sheetId="32" r:id="rId15"/>
+    <sheet name="settings{}depend()" sheetId="29" r:id="rId16"/>
+    <sheet name="ctx" sheetId="22" r:id="rId17"/>
+    <sheet name="Service (ES6)" sheetId="20" r:id="rId18"/>
+    <sheet name="API Gateway" sheetId="18" r:id="rId19"/>
+    <sheet name="Hooks" sheetId="38" r:id="rId20"/>
+    <sheet name="File up(down)load aliases" sheetId="35" r:id="rId21"/>
+    <sheet name="Response type" sheetId="36" r:id="rId22"/>
+    <sheet name="Authorization &amp; Authent" sheetId="37" r:id="rId23"/>
+    <sheet name="Transporter" sheetId="31" r:id="rId24"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="1607">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1931" uniqueCount="1612">
   <si>
     <t>Документация https://moleculer.services/docs/0.14/broker</t>
   </si>
@@ -19005,17 +19006,48 @@
 broker.start();                                     // Запускаем брокер (стартуем все сервисы и подключаемся к транспорту)</t>
     </r>
   </si>
+  <si>
+    <t>DB Adapters</t>
+  </si>
+  <si>
+    <t>`https://moleculer.services/docs/0.15/moleculer-db#Sequelize-Adapter</t>
+  </si>
+  <si>
+    <t>Читать тут:</t>
+  </si>
+  <si>
+    <t>`https://github.com/moleculerjs/moleculer-db/blob/master/packages/moleculer-db-adapter-sequelize/README.md#raw-queries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">github расширенная документация </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="49">
+  <fonts count="51">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -19715,7 +19747,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -19726,23 +19758,23 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -19760,7 +19792,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19778,7 +19810,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19799,7 +19831,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19820,7 +19852,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19838,10 +19870,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19850,28 +19882,28 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19880,49 +19912,49 @@
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="30" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="32" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19931,7 +19963,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19940,7 +19972,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19952,7 +19984,7 @@
     <xf numFmtId="49" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -19961,22 +19993,22 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19988,61 +20020,73 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="30" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -20051,8 +20095,14 @@
     <xf numFmtId="49" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -20060,46 +20110,34 @@
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="33" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="31" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -20108,17 +20146,14 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -21397,6 +21432,730 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{488D8CBB-84D5-4AB1-A098-C4B0F9061CFB}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.39997558519241921"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V34"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="72.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="C3" s="97" t="s">
+        <v>901</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22" s="7" customFormat="1">
+      <c r="A4" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="B4" s="45" t="s">
+        <v>410</v>
+      </c>
+      <c r="C4" s="60"/>
+      <c r="D4" s="12" t="s">
+        <v>404</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="8"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="1"/>
+    </row>
+    <row r="5" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A5" s="1"/>
+      <c r="B5" s="52" t="s">
+        <v>406</v>
+      </c>
+      <c r="C5" s="52" t="s">
+        <v>405</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="1"/>
+    </row>
+    <row r="6" spans="1:22" s="7" customFormat="1" ht="230.4">
+      <c r="A6" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="1"/>
+    </row>
+    <row r="7" spans="1:22" s="7" customFormat="1" ht="43.2">
+      <c r="A7" s="47" t="s">
+        <v>409</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="42" t="s">
+        <v>309</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="1"/>
+    </row>
+    <row r="8" spans="1:22" s="7" customFormat="1" ht="43.2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="1"/>
+    </row>
+    <row r="9" spans="1:22" s="7" customFormat="1" ht="86.4">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C9" s="42" t="s">
+        <v>318</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="1"/>
+    </row>
+    <row r="10" spans="1:22" s="7" customFormat="1">
+      <c r="A10" s="1"/>
+      <c r="B10" s="43" t="s">
+        <v>323</v>
+      </c>
+      <c r="C10" s="43" t="s">
+        <v>324</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="1"/>
+    </row>
+    <row r="11" spans="1:22" s="7" customFormat="1">
+      <c r="A11" s="1"/>
+      <c r="B11" s="42" t="s">
+        <v>325</v>
+      </c>
+      <c r="C11" s="42" t="s">
+        <v>326</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="1"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="1"/>
+    </row>
+    <row r="12" spans="1:22" s="7" customFormat="1">
+      <c r="A12" s="1"/>
+      <c r="B12" s="42" t="s">
+        <v>301</v>
+      </c>
+      <c r="C12" s="42" t="s">
+        <v>327</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="1"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="1"/>
+    </row>
+    <row r="13" spans="1:22" s="7" customFormat="1">
+      <c r="A13" s="1"/>
+      <c r="B13" s="42" t="s">
+        <v>241</v>
+      </c>
+      <c r="C13" s="42" t="s">
+        <v>327</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="1"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="2"/>
+      <c r="V13" s="1"/>
+    </row>
+    <row r="14" spans="1:22" s="7" customFormat="1" ht="28.8">
+      <c r="A14" s="1"/>
+      <c r="B14" s="42" t="s">
+        <v>328</v>
+      </c>
+      <c r="C14" s="42" t="s">
+        <v>329</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="1"/>
+    </row>
+    <row r="15" spans="1:22" s="7" customFormat="1">
+      <c r="A15" s="1"/>
+      <c r="B15" s="42" t="s">
+        <v>330</v>
+      </c>
+      <c r="C15" s="42" t="s">
+        <v>327</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="8"/>
+      <c r="U15" s="2"/>
+      <c r="V15" s="1"/>
+    </row>
+    <row r="16" spans="1:22" s="7" customFormat="1">
+      <c r="A16" s="1"/>
+      <c r="B16" s="42" t="s">
+        <v>331</v>
+      </c>
+      <c r="C16" s="42" t="s">
+        <v>326</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="8"/>
+      <c r="U16" s="2"/>
+      <c r="V16" s="1"/>
+    </row>
+    <row r="17" spans="1:22" s="7" customFormat="1">
+      <c r="A17" s="1"/>
+      <c r="B17" s="42" t="s">
+        <v>332</v>
+      </c>
+      <c r="C17" s="42" t="s">
+        <v>333</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="8"/>
+      <c r="U17" s="2"/>
+      <c r="V17" s="1"/>
+    </row>
+    <row r="18" spans="1:22" s="7" customFormat="1">
+      <c r="A18" s="1"/>
+      <c r="B18" s="42" t="s">
+        <v>334</v>
+      </c>
+      <c r="C18" s="42" t="s">
+        <v>333</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="1"/>
+      <c r="T18" s="8"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="1"/>
+    </row>
+    <row r="19" spans="1:22" s="7" customFormat="1">
+      <c r="A19" s="1"/>
+      <c r="B19" s="42" t="s">
+        <v>308</v>
+      </c>
+      <c r="C19" s="42" t="s">
+        <v>326</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="8"/>
+      <c r="U19" s="2"/>
+      <c r="V19" s="1"/>
+    </row>
+    <row r="20" spans="1:22" s="7" customFormat="1">
+      <c r="A20" s="1"/>
+      <c r="B20" s="42" t="s">
+        <v>335</v>
+      </c>
+      <c r="C20" s="42" t="s">
+        <v>326</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="8"/>
+      <c r="U20" s="2"/>
+      <c r="V20" s="1"/>
+    </row>
+    <row r="21" spans="1:22" s="7" customFormat="1">
+      <c r="A21" s="1"/>
+      <c r="B21" s="42" t="s">
+        <v>336</v>
+      </c>
+      <c r="C21" s="42" t="s">
+        <v>326</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="1"/>
+      <c r="T21" s="8"/>
+      <c r="U21" s="2"/>
+      <c r="V21" s="1"/>
+    </row>
+    <row r="22" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A22" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B22" s="42" t="s">
+        <v>313</v>
+      </c>
+      <c r="C22" s="42" t="s">
+        <v>311</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2"/>
+      <c r="S22" s="1"/>
+      <c r="T22" s="8"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="1"/>
+    </row>
+    <row r="23" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A23" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="B23" s="42" t="s">
+        <v>314</v>
+      </c>
+      <c r="C23" s="42" t="s">
+        <v>312</v>
+      </c>
+      <c r="D23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="8"/>
+      <c r="U23" s="2"/>
+      <c r="V23" s="1"/>
+    </row>
+    <row r="24" spans="1:22" s="7" customFormat="1">
+      <c r="A24" s="55" t="s">
+        <v>412</v>
+      </c>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="1"/>
+      <c r="T24" s="8"/>
+      <c r="U24" s="2"/>
+      <c r="V24" s="1"/>
+    </row>
+    <row r="25" spans="1:22" s="7" customFormat="1" ht="144">
+      <c r="A25" s="1"/>
+      <c r="B25" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="D25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="1"/>
+      <c r="T25" s="8"/>
+      <c r="U25" s="2"/>
+      <c r="V25" s="1"/>
+    </row>
+    <row r="26" spans="1:22" s="7" customFormat="1">
+      <c r="A26" s="55" t="s">
+        <v>321</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="P26" s="2"/>
+      <c r="Q26" s="2"/>
+      <c r="R26" s="2"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="8"/>
+      <c r="U26" s="2"/>
+      <c r="V26" s="1"/>
+    </row>
+    <row r="27" spans="1:22" s="7" customFormat="1" ht="57.6">
+      <c r="A27" s="1"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="42" t="s">
+        <v>322</v>
+      </c>
+      <c r="D27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="P27" s="2"/>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
+      <c r="S27" s="1"/>
+      <c r="T27" s="8"/>
+      <c r="U27" s="2"/>
+      <c r="V27" s="1"/>
+    </row>
+    <row r="28" spans="1:22">
+      <c r="A28" s="3"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="P28" s="5"/>
+      <c r="Q28" s="5"/>
+      <c r="R28" s="5"/>
+      <c r="S28" s="5"/>
+      <c r="U28" s="5"/>
+    </row>
+    <row r="29" spans="1:22">
+      <c r="C29" s="97" t="s">
+        <v>1109</v>
+      </c>
+      <c r="P29" s="1"/>
+      <c r="U29" s="1"/>
+      <c r="V29" s="2"/>
+    </row>
+    <row r="30" spans="1:22" ht="28.8">
+      <c r="C30" s="95" t="s">
+        <v>1110</v>
+      </c>
+      <c r="P30" s="1"/>
+      <c r="U30" s="1"/>
+      <c r="V30" s="2"/>
+    </row>
+    <row r="31" spans="1:22">
+      <c r="A31" s="47" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" ht="244.8">
+      <c r="C32" s="95" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="47" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="187.2">
+      <c r="C34" s="95" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03D965FF-3469-4ADC-BFBB-2C499831567E}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -22254,7 +23013,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D88F61F-8C7C-4710-8F38-D46F66310E17}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -22486,7 +23245,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7C45E35-A0E9-4FBE-88F3-CE4B282CF0DD}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -23641,7 +24400,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F722A6B-FDD4-4F28-A73E-E1B84FE9A13E}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -24405,7 +25164,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2EDDD90-7CFC-46CE-93A4-19D76FB6A77B}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -24833,7 +25592,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF050F64-E219-48FB-BA24-6D9B0B37599F}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -25174,7 +25933,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9400A441-6B67-47CF-87A5-3C3813CBCD51}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -25554,7 +26313,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C7DACD-972C-4F9B-8B6E-158B3A84F36B}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -25670,7 +26429,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B84D070D-9F43-498E-8C8B-DA56F9B43AEF}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -27760,313 +28519,7 @@
       <c r="V87" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="23" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{215A08A6-8FA5-47FE-AD3E-099EDF44B417}">
-  <sheetPr>
-    <tabColor theme="4" tint="-0.249977111117893"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A2:V40"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="41.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" style="8"/>
-    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.77734375" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:22">
-      <c r="A2" s="3"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="U2" s="5"/>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="C3" s="116" t="s">
-        <v>1468</v>
-      </c>
-      <c r="P3" s="1"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:22">
-      <c r="C4" s="115" t="s">
-        <v>1469</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>1476</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22">
-      <c r="C5" s="115" t="s">
-        <v>1470</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22">
-      <c r="C6" s="115" t="s">
-        <v>1302</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22">
-      <c r="C7" s="115" t="s">
-        <v>1303</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22">
-      <c r="C8" s="115" t="s">
-        <v>1471</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22">
-      <c r="C9" s="115" t="s">
-        <v>1472</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>1497</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22">
-      <c r="C10" s="115" t="s">
-        <v>1473</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22">
-      <c r="C11" s="115" t="s">
-        <v>1474</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>1475</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22">
-      <c r="A13" s="118" t="s">
-        <v>1469</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>1476</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22" ht="28.8">
-      <c r="C14" s="115" t="s">
-        <v>1479</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" ht="302.39999999999998">
-      <c r="C15" s="115" t="s">
-        <v>1482</v>
-      </c>
-    </row>
-    <row r="16" spans="1:22">
-      <c r="A16" s="12" t="s">
-        <v>1470</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>1477</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="C17" s="115" t="s">
-        <v>1480</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="331.2">
-      <c r="B18" s="2" t="s">
-        <v>1483</v>
-      </c>
-      <c r="C18" s="115" t="s">
-        <v>1481</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="12" t="s">
-        <v>1302</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>1478</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="28.8">
-      <c r="C20" s="115" t="s">
-        <v>1484</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="302.39999999999998">
-      <c r="C21" s="115" t="s">
-        <v>1485</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="172.8">
-      <c r="C22" s="115" t="s">
-        <v>1486</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="12" t="s">
-        <v>1303</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="409.6">
-      <c r="A24" s="131" t="s">
-        <v>1540</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>1488</v>
-      </c>
-      <c r="C24" s="131" t="s">
-        <v>1487</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="12" t="s">
-        <v>1471</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>1491</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="129.6">
-      <c r="B26" s="2" t="s">
-        <v>1494</v>
-      </c>
-      <c r="C26" s="115" t="s">
-        <v>1489</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="230.4">
-      <c r="B27" s="2" t="s">
-        <v>1492</v>
-      </c>
-      <c r="C27" s="115" t="s">
-        <v>1490</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>1493</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="12" t="s">
-        <v>1472</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>1497</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="28.8">
-      <c r="C29" s="115" t="s">
-        <v>1496</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="244.8">
-      <c r="C30" s="115" t="s">
-        <v>1495</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="12" t="s">
-        <v>1498</v>
-      </c>
-      <c r="C31" s="1"/>
-    </row>
-    <row r="32" spans="1:4" ht="43.2">
-      <c r="A32" s="2"/>
-      <c r="C32" s="115" t="s">
-        <v>1505</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="86.4">
-      <c r="A33" s="2" t="s">
-        <v>1506</v>
-      </c>
-      <c r="C33" s="115" t="s">
-        <v>1507</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="2"/>
-      <c r="C34" s="115"/>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" s="119" t="s">
-        <v>1316</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="C36" s="115" t="s">
-        <v>1499</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" s="13" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="129.6">
-      <c r="C38" s="115" t="s">
-        <v>1501</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="244.8">
-      <c r="A39" s="1" t="s">
-        <v>1502</v>
-      </c>
-      <c r="C39" s="115" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="288">
-      <c r="A40" s="1" t="s">
-        <v>1504</v>
-      </c>
-      <c r="C40" s="115" t="s">
-        <v>1500</v>
-      </c>
-    </row>
-  </sheetData>
+  <phoneticPr fontId="25" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -28335,13 +28788,319 @@
       <c r="D25" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="23" type="noConversion"/>
+  <phoneticPr fontId="25" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{215A08A6-8FA5-47FE-AD3E-099EDF44B417}">
+  <sheetPr>
+    <tabColor theme="4" tint="-0.249977111117893"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V40"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="41.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3" s="116" t="s">
+        <v>1468</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22">
+      <c r="C4" s="115" t="s">
+        <v>1469</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22">
+      <c r="C5" s="115" t="s">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22">
+      <c r="C6" s="115" t="s">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22">
+      <c r="C7" s="115" t="s">
+        <v>1303</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22">
+      <c r="C8" s="115" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22">
+      <c r="C9" s="115" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>1497</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22">
+      <c r="C10" s="115" t="s">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22">
+      <c r="C11" s="115" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
+      <c r="A13" s="118" t="s">
+        <v>1469</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="28.8">
+      <c r="C14" s="115" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="302.39999999999998">
+      <c r="C15" s="115" t="s">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22">
+      <c r="A16" s="12" t="s">
+        <v>1470</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>1477</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="C17" s="115" t="s">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="331.2">
+      <c r="B18" s="2" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C18" s="115" t="s">
+        <v>1481</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="12" t="s">
+        <v>1302</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>1478</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="28.8">
+      <c r="C20" s="115" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="302.39999999999998">
+      <c r="C21" s="115" t="s">
+        <v>1485</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="172.8">
+      <c r="C22" s="115" t="s">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="12" t="s">
+        <v>1303</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="409.6">
+      <c r="A24" s="131" t="s">
+        <v>1540</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>1488</v>
+      </c>
+      <c r="C24" s="131" t="s">
+        <v>1487</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="12" t="s">
+        <v>1471</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="129.6">
+      <c r="B26" s="2" t="s">
+        <v>1494</v>
+      </c>
+      <c r="C26" s="115" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="230.4">
+      <c r="B27" s="2" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C27" s="115" t="s">
+        <v>1490</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>1493</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="12" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>1497</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="28.8">
+      <c r="C29" s="115" t="s">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="244.8">
+      <c r="C30" s="115" t="s">
+        <v>1495</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="12" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C31" s="1"/>
+    </row>
+    <row r="32" spans="1:4" ht="43.2">
+      <c r="A32" s="2"/>
+      <c r="C32" s="115" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="86.4">
+      <c r="A33" s="2" t="s">
+        <v>1506</v>
+      </c>
+      <c r="C33" s="115" t="s">
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="2"/>
+      <c r="C34" s="115"/>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="119" t="s">
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="C36" s="115" t="s">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="13" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="129.6">
+      <c r="C38" s="115" t="s">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="244.8">
+      <c r="A39" s="1" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C39" s="115" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="288">
+      <c r="A40" s="1" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C40" s="115" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E63D7CF-A8C1-4EE2-B24F-BB6423312324}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -28483,7 +29242,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0E1A7F4-4156-43BA-A471-45FED5CB2B12}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -28631,7 +29390,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC0D01A-891F-4564-985B-BABA4F41741B}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -28765,7 +29524,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C83401B-1940-4C7B-967F-92D40F8BF33D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -28972,6 +29731,218 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C71290A-1585-4566-B486-FCA71E7E03ED}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:V9"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="8"/>
+    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:22">
+      <c r="A2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="U2" s="5"/>
+    </row>
+    <row r="3" spans="1:22">
+      <c r="A3" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C3" s="137" t="s">
+        <v>1607</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>1040</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22" s="7" customFormat="1">
+      <c r="A4" s="12" t="s">
+        <v>1607</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="8"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="1"/>
+    </row>
+    <row r="5" spans="1:22" s="7" customFormat="1">
+      <c r="A5" s="1"/>
+      <c r="B5" s="2" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>1608</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="1"/>
+    </row>
+    <row r="6" spans="1:22" s="7" customFormat="1" ht="28.8">
+      <c r="A6" s="1"/>
+      <c r="B6" s="2" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>1610</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="1"/>
+    </row>
+    <row r="7" spans="1:22" s="7" customFormat="1">
+      <c r="A7" s="1"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="52"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="1"/>
+    </row>
+    <row r="8" spans="1:22" s="7" customFormat="1">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="1"/>
+    </row>
+    <row r="9" spans="1:22" s="7" customFormat="1">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11C0BAE5-4B5A-4ED9-9078-DE65AE578F59}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -29125,7 +30096,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA45549C-F4E3-4DE8-8796-B64020ED8004}">
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
@@ -29559,7 +30530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC501503-0164-402D-9D9C-86B5F52AE94D}">
   <sheetPr>
     <tabColor theme="1"/>
@@ -30384,7 +31355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{948CE0B5-C565-4729-8A1A-36CD87669389}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -31057,7 +32028,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53293E74-C56C-43CE-8332-3FF6CCF78D58}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -33147,7 +34118,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47DCDB03-35F5-4E59-94D1-F4F42160A968}">
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
@@ -35226,728 +36197,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{488D8CBB-84D5-4AB1-A098-C4B0F9061CFB}">
-  <sheetPr>
-    <tabColor theme="5" tint="0.39997558519241921"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A2:V34"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="72.21875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.21875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.77734375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.77734375" style="7" customWidth="1"/>
-    <col min="16" max="16" width="56.77734375" style="2" customWidth="1"/>
-    <col min="17" max="17" width="46.77734375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="62.88671875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.77734375" style="8"/>
-    <col min="21" max="21" width="67.77734375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.77734375" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:22">
-      <c r="A2" s="3"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="U2" s="5"/>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="C3" s="97" t="s">
-        <v>901</v>
-      </c>
-      <c r="P3" s="1"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:22" s="7" customFormat="1">
-      <c r="A4" s="12" t="s">
-        <v>308</v>
-      </c>
-      <c r="B4" s="45" t="s">
-        <v>410</v>
-      </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="12" t="s">
-        <v>404</v>
-      </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="1"/>
-      <c r="T4" s="8"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="1"/>
-    </row>
-    <row r="5" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A5" s="1"/>
-      <c r="B5" s="52" t="s">
-        <v>406</v>
-      </c>
-      <c r="C5" s="52" t="s">
-        <v>405</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="1"/>
-    </row>
-    <row r="6" spans="1:22" s="7" customFormat="1" ht="230.4">
-      <c r="A6" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="8"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="1"/>
-    </row>
-    <row r="7" spans="1:22" s="7" customFormat="1" ht="43.2">
-      <c r="A7" s="47" t="s">
-        <v>409</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="42" t="s">
-        <v>309</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="8"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="1"/>
-    </row>
-    <row r="8" spans="1:22" s="7" customFormat="1" ht="43.2">
-      <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="42" t="s">
-        <v>310</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="1"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="1"/>
-    </row>
-    <row r="9" spans="1:22" s="7" customFormat="1" ht="86.4">
-      <c r="A9" s="1"/>
-      <c r="B9" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="C9" s="42" t="s">
-        <v>318</v>
-      </c>
-      <c r="D9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="8"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="1"/>
-    </row>
-    <row r="10" spans="1:22" s="7" customFormat="1">
-      <c r="A10" s="1"/>
-      <c r="B10" s="43" t="s">
-        <v>323</v>
-      </c>
-      <c r="C10" s="43" t="s">
-        <v>324</v>
-      </c>
-      <c r="D10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="1"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="1"/>
-    </row>
-    <row r="11" spans="1:22" s="7" customFormat="1">
-      <c r="A11" s="1"/>
-      <c r="B11" s="42" t="s">
-        <v>325</v>
-      </c>
-      <c r="C11" s="42" t="s">
-        <v>326</v>
-      </c>
-      <c r="D11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="1"/>
-      <c r="T11" s="8"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="1"/>
-    </row>
-    <row r="12" spans="1:22" s="7" customFormat="1">
-      <c r="A12" s="1"/>
-      <c r="B12" s="42" t="s">
-        <v>301</v>
-      </c>
-      <c r="C12" s="42" t="s">
-        <v>327</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="1"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="2"/>
-      <c r="V12" s="1"/>
-    </row>
-    <row r="13" spans="1:22" s="7" customFormat="1">
-      <c r="A13" s="1"/>
-      <c r="B13" s="42" t="s">
-        <v>241</v>
-      </c>
-      <c r="C13" s="42" t="s">
-        <v>327</v>
-      </c>
-      <c r="D13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="1"/>
-    </row>
-    <row r="14" spans="1:22" s="7" customFormat="1" ht="28.8">
-      <c r="A14" s="1"/>
-      <c r="B14" s="42" t="s">
-        <v>328</v>
-      </c>
-      <c r="C14" s="42" t="s">
-        <v>329</v>
-      </c>
-      <c r="D14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="8"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="1"/>
-    </row>
-    <row r="15" spans="1:22" s="7" customFormat="1">
-      <c r="A15" s="1"/>
-      <c r="B15" s="42" t="s">
-        <v>330</v>
-      </c>
-      <c r="C15" s="42" t="s">
-        <v>327</v>
-      </c>
-      <c r="D15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="1"/>
-      <c r="T15" s="8"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="1"/>
-    </row>
-    <row r="16" spans="1:22" s="7" customFormat="1">
-      <c r="A16" s="1"/>
-      <c r="B16" s="42" t="s">
-        <v>331</v>
-      </c>
-      <c r="C16" s="42" t="s">
-        <v>326</v>
-      </c>
-      <c r="D16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="8"/>
-      <c r="U16" s="2"/>
-      <c r="V16" s="1"/>
-    </row>
-    <row r="17" spans="1:22" s="7" customFormat="1">
-      <c r="A17" s="1"/>
-      <c r="B17" s="42" t="s">
-        <v>332</v>
-      </c>
-      <c r="C17" s="42" t="s">
-        <v>333</v>
-      </c>
-      <c r="D17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="8"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="1"/>
-    </row>
-    <row r="18" spans="1:22" s="7" customFormat="1">
-      <c r="A18" s="1"/>
-      <c r="B18" s="42" t="s">
-        <v>334</v>
-      </c>
-      <c r="C18" s="42" t="s">
-        <v>333</v>
-      </c>
-      <c r="D18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="8"/>
-      <c r="U18" s="2"/>
-      <c r="V18" s="1"/>
-    </row>
-    <row r="19" spans="1:22" s="7" customFormat="1">
-      <c r="A19" s="1"/>
-      <c r="B19" s="42" t="s">
-        <v>308</v>
-      </c>
-      <c r="C19" s="42" t="s">
-        <v>326</v>
-      </c>
-      <c r="D19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="8"/>
-      <c r="U19" s="2"/>
-      <c r="V19" s="1"/>
-    </row>
-    <row r="20" spans="1:22" s="7" customFormat="1">
-      <c r="A20" s="1"/>
-      <c r="B20" s="42" t="s">
-        <v>335</v>
-      </c>
-      <c r="C20" s="42" t="s">
-        <v>326</v>
-      </c>
-      <c r="D20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="8"/>
-      <c r="U20" s="2"/>
-      <c r="V20" s="1"/>
-    </row>
-    <row r="21" spans="1:22" s="7" customFormat="1">
-      <c r="A21" s="1"/>
-      <c r="B21" s="42" t="s">
-        <v>336</v>
-      </c>
-      <c r="C21" s="42" t="s">
-        <v>326</v>
-      </c>
-      <c r="D21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="8"/>
-      <c r="U21" s="2"/>
-      <c r="V21" s="1"/>
-    </row>
-    <row r="22" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A22" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="B22" s="42" t="s">
-        <v>313</v>
-      </c>
-      <c r="C22" s="42" t="s">
-        <v>311</v>
-      </c>
-      <c r="D22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="8"/>
-      <c r="U22" s="2"/>
-      <c r="V22" s="1"/>
-    </row>
-    <row r="23" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A23" s="1" t="s">
-        <v>315</v>
-      </c>
-      <c r="B23" s="42" t="s">
-        <v>314</v>
-      </c>
-      <c r="C23" s="42" t="s">
-        <v>312</v>
-      </c>
-      <c r="D23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="8"/>
-      <c r="U23" s="2"/>
-      <c r="V23" s="1"/>
-    </row>
-    <row r="24" spans="1:22" s="7" customFormat="1">
-      <c r="A24" s="55" t="s">
-        <v>412</v>
-      </c>
-      <c r="B24" s="42"/>
-      <c r="C24" s="42"/>
-      <c r="D24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="1"/>
-      <c r="T24" s="8"/>
-      <c r="U24" s="2"/>
-      <c r="V24" s="1"/>
-    </row>
-    <row r="25" spans="1:22" s="7" customFormat="1" ht="144">
-      <c r="A25" s="1"/>
-      <c r="B25" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="D25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="2"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="8"/>
-      <c r="U25" s="2"/>
-      <c r="V25" s="1"/>
-    </row>
-    <row r="26" spans="1:22" s="7" customFormat="1">
-      <c r="A26" s="55" t="s">
-        <v>321</v>
-      </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
-      <c r="P26" s="2"/>
-      <c r="Q26" s="2"/>
-      <c r="R26" s="2"/>
-      <c r="S26" s="1"/>
-      <c r="T26" s="8"/>
-      <c r="U26" s="2"/>
-      <c r="V26" s="1"/>
-    </row>
-    <row r="27" spans="1:22" s="7" customFormat="1" ht="57.6">
-      <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="42" t="s">
-        <v>322</v>
-      </c>
-      <c r="D27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-      <c r="K27" s="1"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="P27" s="2"/>
-      <c r="Q27" s="2"/>
-      <c r="R27" s="2"/>
-      <c r="S27" s="1"/>
-      <c r="T27" s="8"/>
-      <c r="U27" s="2"/>
-      <c r="V27" s="1"/>
-    </row>
-    <row r="28" spans="1:22">
-      <c r="A28" s="3"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="P28" s="5"/>
-      <c r="Q28" s="5"/>
-      <c r="R28" s="5"/>
-      <c r="S28" s="5"/>
-      <c r="U28" s="5"/>
-    </row>
-    <row r="29" spans="1:22">
-      <c r="C29" s="97" t="s">
-        <v>1109</v>
-      </c>
-      <c r="P29" s="1"/>
-      <c r="U29" s="1"/>
-      <c r="V29" s="2"/>
-    </row>
-    <row r="30" spans="1:22" ht="28.8">
-      <c r="C30" s="95" t="s">
-        <v>1110</v>
-      </c>
-      <c r="P30" s="1"/>
-      <c r="U30" s="1"/>
-      <c r="V30" s="2"/>
-    </row>
-    <row r="31" spans="1:22">
-      <c r="A31" s="47" t="s">
-        <v>1105</v>
-      </c>
-    </row>
-    <row r="32" spans="1:22" ht="244.8">
-      <c r="C32" s="95" t="s">
-        <v>1111</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" s="47" t="s">
-        <v>1106</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="187.2">
-      <c r="C34" s="95" t="s">
-        <v>1107</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>